<commit_message>
W03 SAT workbooks after the rigor and pedagogy reviews: the grade closure workbook flags a seat whose group part differs from a teammate's and refuses ABSENT in the group part, since every member receives the group's 34; both workbooks leave a demo recovered inside its two minutes to the panel's judgement instead of counting it as run cold; the Read me sheets drop process words; three new flips in the closure manifest and one in the scoring manifest, all recalculated through LibreOffice; the run sheet's closure step clears the new flag
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VFn7PXPJsRCn9QfcoxZL6T
</commit_message>
<xml_diff>
--- a/content/W03/SAT/rubrics/C2_W03_SAT_grade_closure_TRAINER.xlsx
+++ b/content/W03/SAT/rubrics/C2_W03_SAT_grade_closure_TRAINER.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>COMPLETE when all four scores are in, within their maximums and within the demo rule. NOT A SCORE means text other than ABSENT, or a negative number. OVER MAX means a score above its maximum. DEMO RULE means full marks on presentation and defence for a group whose demo still failed. MISSING names the scores still to enter. ABSENT names the events the learner missed when every other score is in.</t>
+          <t>COMPLETE when all four scores are in, within their maximums and within the demo rule. NOT A SCORE means text other than ABSENT, ABSENT typed in the group part (which every member receives), or a negative number. OVER MAX means a score above its maximum. GROUP PART DIFFERS means this seat's group part is not the same number as a teammate's; the panel scored the group once, so one of the copies is wrong. DEMO RULE means full marks on presentation and defence for a group whose demo still failed. MISSING names the scores still to enter. ABSENT names the events the learner missed when every other score is in.</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>A learner who missed an event has ABSENT typed in that event's cell and the Programme Head's decision in Notes. The seat then counts as closed, carries no total, and is listed on the Checks sheet. No make-up rule is published, so this workbook sets none.</t>
+          <t>A learner who missed an event has ABSENT typed in that event's cell and the Programme Head's decision in Notes. For the mini project, ABSENT goes in the presentation and defence cell; the group part stays the group's number, since the rubric gives every member the 34. The seat then counts as closed, carries no total, and is listed on the Checks sheet. No make-up rule is published, so this workbook sets none.</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="B4" s="10" t="n"/>
       <c r="C4" s="9">
-        <f>IF(B4="","record the outcome from the scoring sheet",IF(B4="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B4="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B4="","record the outcome from the scoring sheet",IF(B4="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B4="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B4="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="B5" s="10" t="n"/>
       <c r="C5" s="9">
-        <f>IF(B5="","record the outcome from the scoring sheet",IF(B5="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B5="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B5="","record the outcome from the scoring sheet",IF(B5="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B5="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B5="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="B6" s="10" t="n"/>
       <c r="C6" s="9">
-        <f>IF(B6="","record the outcome from the scoring sheet",IF(B6="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B6="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B6="","record the outcome from the scoring sheet",IF(B6="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B6="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B6="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="9">
-        <f>IF(B7="","record the outcome from the scoring sheet",IF(B7="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B7="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B7="","record the outcome from the scoring sheet",IF(B7="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B7="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B7="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B8" s="10" t="n"/>
       <c r="C8" s="9">
-        <f>IF(B8="","record the outcome from the scoring sheet",IF(B8="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B8="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B8="","record the outcome from the scoring sheet",IF(B8="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B8="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B8="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="B9" s="10" t="n"/>
       <c r="C9" s="9">
-        <f>IF(B9="","record the outcome from the scoring sheet",IF(B9="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B9="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B9="","record the outcome from the scoring sheet",IF(B9="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B9="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B9="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="B10" s="10" t="n"/>
       <c r="C10" s="9">
-        <f>IF(B10="","record the outcome from the scoring sheet",IF(B10="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B10="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B10="","record the outcome from the scoring sheet",IF(B10="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B10="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B10="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="B11" s="10" t="n"/>
       <c r="C11" s="9">
-        <f>IF(B11="","record the outcome from the scoring sheet",IF(B11="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B11="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B11="","record the outcome from the scoring sheet",IF(B11="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B11="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B11="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="9">
-        <f>IF(B12="","record the outcome from the scoring sheet",IF(B12="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B12="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first","no change: the live demo counts as run cold")))</f>
+        <f>IF(B12="","record the outcome from the scoring sheet",IF(B12="still failed: presented from the executed notebook","the group's 34 stand on the executed run; presentation and defence cannot be full marks",IF(B12="machine failed: demo waits for the reserve","not final: the demo runs cold in the reserve first",IF(B12="recovered within two minutes","the rule sets nothing for a recovery: the panel judged it within presentation and defence","no change: the live demo ran cold"))))</f>
         <v/>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
         <v/>
       </c>
       <c r="L6" s="9">
-        <f>IF(OR(AND(E6&lt;&gt;"",NOT(ISNUMBER(E6)),E6&lt;&gt;"ABSENT"),AND(F6&lt;&gt;"",NOT(ISNUMBER(F6)),F6&lt;&gt;"ABSENT"),AND(G6&lt;&gt;"",NOT(ISNUMBER(G6)),G6&lt;&gt;"ABSENT"),AND(H6&lt;&gt;"",NOT(ISNUMBER(H6)),H6&lt;&gt;"ABSENT"),AND(ISNUMBER(E6),E6&lt;0),AND(ISNUMBER(F6),F6&lt;0),AND(ISNUMBER(G6),G6&lt;0),AND(ISNUMBER(H6),H6&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E6),E6&gt;E$4),AND(ISNUMBER(F6),F6&gt;F$4),AND(ISNUMBER(G6),G6&gt;G$4),AND(ISNUMBER(H6),H6&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G6),K6="still failed: presented from the executed notebook",G6&gt;=$G$4),"DEMO RULE",IF(COUNT(E6:H6)+COUNTIF(E6:H6,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E6="","GD ","")&amp;IF(F6="","group part ","")&amp;IF(G6="","presentation and defence ","")&amp;IF(H6="","mock","")),IF(COUNTIF(E6:H6,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E6="ABSENT","GD ","")&amp;IF(F6="ABSENT","group part ","")&amp;IF(G6="ABSENT","presentation and defence ","")&amp;IF(H6="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E6&lt;&gt;"",NOT(ISNUMBER(E6)),E6&lt;&gt;"ABSENT"),AND(F6&lt;&gt;"",NOT(ISNUMBER(F6)),F6&lt;&gt;"ABSENT"),AND(G6&lt;&gt;"",NOT(ISNUMBER(G6)),G6&lt;&gt;"ABSENT"),AND(H6&lt;&gt;"",NOT(ISNUMBER(H6)),H6&lt;&gt;"ABSENT"),AND(F6&lt;&gt;"",NOT(ISNUMBER(F6))),AND(ISNUMBER(E6),E6&lt;0),AND(ISNUMBER(F6),F6&lt;0),AND(ISNUMBER(G6),G6&lt;0),AND(ISNUMBER(H6),H6&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E6),E6&gt;E$4),AND(ISNUMBER(F6),F6&gt;F$4),AND(ISNUMBER(G6),G6&gt;G$4),AND(ISNUMBER(H6),H6&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F6),SUMPRODUCT(($B$6:$B$40=B6)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F6))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G6),K6="still failed: presented from the executed notebook",G6&gt;=$G$4),"DEMO RULE",IF(COUNT(E6:H6)+COUNTIF(E6:H6,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E6="","GD ","")&amp;IF(F6="","group part ","")&amp;IF(G6="","presentation and defence ","")&amp;IF(H6="","mock","")),IF(COUNTIF(E6:H6,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E6="ABSENT","GD ","")&amp;IF(F6="ABSENT","group part ","")&amp;IF(G6="ABSENT","presentation and defence ","")&amp;IF(H6="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M6" s="10" t="n"/>
@@ -1285,7 +1285,7 @@
         <v/>
       </c>
       <c r="L7" s="9">
-        <f>IF(OR(AND(E7&lt;&gt;"",NOT(ISNUMBER(E7)),E7&lt;&gt;"ABSENT"),AND(F7&lt;&gt;"",NOT(ISNUMBER(F7)),F7&lt;&gt;"ABSENT"),AND(G7&lt;&gt;"",NOT(ISNUMBER(G7)),G7&lt;&gt;"ABSENT"),AND(H7&lt;&gt;"",NOT(ISNUMBER(H7)),H7&lt;&gt;"ABSENT"),AND(ISNUMBER(E7),E7&lt;0),AND(ISNUMBER(F7),F7&lt;0),AND(ISNUMBER(G7),G7&lt;0),AND(ISNUMBER(H7),H7&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E7),E7&gt;E$4),AND(ISNUMBER(F7),F7&gt;F$4),AND(ISNUMBER(G7),G7&gt;G$4),AND(ISNUMBER(H7),H7&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G7),K7="still failed: presented from the executed notebook",G7&gt;=$G$4),"DEMO RULE",IF(COUNT(E7:H7)+COUNTIF(E7:H7,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E7="","GD ","")&amp;IF(F7="","group part ","")&amp;IF(G7="","presentation and defence ","")&amp;IF(H7="","mock","")),IF(COUNTIF(E7:H7,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E7="ABSENT","GD ","")&amp;IF(F7="ABSENT","group part ","")&amp;IF(G7="ABSENT","presentation and defence ","")&amp;IF(H7="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E7&lt;&gt;"",NOT(ISNUMBER(E7)),E7&lt;&gt;"ABSENT"),AND(F7&lt;&gt;"",NOT(ISNUMBER(F7)),F7&lt;&gt;"ABSENT"),AND(G7&lt;&gt;"",NOT(ISNUMBER(G7)),G7&lt;&gt;"ABSENT"),AND(H7&lt;&gt;"",NOT(ISNUMBER(H7)),H7&lt;&gt;"ABSENT"),AND(F7&lt;&gt;"",NOT(ISNUMBER(F7))),AND(ISNUMBER(E7),E7&lt;0),AND(ISNUMBER(F7),F7&lt;0),AND(ISNUMBER(G7),G7&lt;0),AND(ISNUMBER(H7),H7&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E7),E7&gt;E$4),AND(ISNUMBER(F7),F7&gt;F$4),AND(ISNUMBER(G7),G7&gt;G$4),AND(ISNUMBER(H7),H7&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F7),SUMPRODUCT(($B$6:$B$40=B7)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F7))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G7),K7="still failed: presented from the executed notebook",G7&gt;=$G$4),"DEMO RULE",IF(COUNT(E7:H7)+COUNTIF(E7:H7,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E7="","GD ","")&amp;IF(F7="","group part ","")&amp;IF(G7="","presentation and defence ","")&amp;IF(H7="","mock","")),IF(COUNTIF(E7:H7,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E7="ABSENT","GD ","")&amp;IF(F7="ABSENT","group part ","")&amp;IF(G7="ABSENT","presentation and defence ","")&amp;IF(H7="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M7" s="10" t="n"/>
@@ -1328,7 +1328,7 @@
         <v/>
       </c>
       <c r="L8" s="9">
-        <f>IF(OR(AND(E8&lt;&gt;"",NOT(ISNUMBER(E8)),E8&lt;&gt;"ABSENT"),AND(F8&lt;&gt;"",NOT(ISNUMBER(F8)),F8&lt;&gt;"ABSENT"),AND(G8&lt;&gt;"",NOT(ISNUMBER(G8)),G8&lt;&gt;"ABSENT"),AND(H8&lt;&gt;"",NOT(ISNUMBER(H8)),H8&lt;&gt;"ABSENT"),AND(ISNUMBER(E8),E8&lt;0),AND(ISNUMBER(F8),F8&lt;0),AND(ISNUMBER(G8),G8&lt;0),AND(ISNUMBER(H8),H8&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E8),E8&gt;E$4),AND(ISNUMBER(F8),F8&gt;F$4),AND(ISNUMBER(G8),G8&gt;G$4),AND(ISNUMBER(H8),H8&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G8),K8="still failed: presented from the executed notebook",G8&gt;=$G$4),"DEMO RULE",IF(COUNT(E8:H8)+COUNTIF(E8:H8,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E8="","GD ","")&amp;IF(F8="","group part ","")&amp;IF(G8="","presentation and defence ","")&amp;IF(H8="","mock","")),IF(COUNTIF(E8:H8,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E8="ABSENT","GD ","")&amp;IF(F8="ABSENT","group part ","")&amp;IF(G8="ABSENT","presentation and defence ","")&amp;IF(H8="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E8&lt;&gt;"",NOT(ISNUMBER(E8)),E8&lt;&gt;"ABSENT"),AND(F8&lt;&gt;"",NOT(ISNUMBER(F8)),F8&lt;&gt;"ABSENT"),AND(G8&lt;&gt;"",NOT(ISNUMBER(G8)),G8&lt;&gt;"ABSENT"),AND(H8&lt;&gt;"",NOT(ISNUMBER(H8)),H8&lt;&gt;"ABSENT"),AND(F8&lt;&gt;"",NOT(ISNUMBER(F8))),AND(ISNUMBER(E8),E8&lt;0),AND(ISNUMBER(F8),F8&lt;0),AND(ISNUMBER(G8),G8&lt;0),AND(ISNUMBER(H8),H8&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E8),E8&gt;E$4),AND(ISNUMBER(F8),F8&gt;F$4),AND(ISNUMBER(G8),G8&gt;G$4),AND(ISNUMBER(H8),H8&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F8),SUMPRODUCT(($B$6:$B$40=B8)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F8))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G8),K8="still failed: presented from the executed notebook",G8&gt;=$G$4),"DEMO RULE",IF(COUNT(E8:H8)+COUNTIF(E8:H8,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E8="","GD ","")&amp;IF(F8="","group part ","")&amp;IF(G8="","presentation and defence ","")&amp;IF(H8="","mock","")),IF(COUNTIF(E8:H8,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E8="ABSENT","GD ","")&amp;IF(F8="ABSENT","group part ","")&amp;IF(G8="ABSENT","presentation and defence ","")&amp;IF(H8="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M8" s="10" t="n"/>
@@ -1371,7 +1371,7 @@
         <v/>
       </c>
       <c r="L9" s="9">
-        <f>IF(OR(AND(E9&lt;&gt;"",NOT(ISNUMBER(E9)),E9&lt;&gt;"ABSENT"),AND(F9&lt;&gt;"",NOT(ISNUMBER(F9)),F9&lt;&gt;"ABSENT"),AND(G9&lt;&gt;"",NOT(ISNUMBER(G9)),G9&lt;&gt;"ABSENT"),AND(H9&lt;&gt;"",NOT(ISNUMBER(H9)),H9&lt;&gt;"ABSENT"),AND(ISNUMBER(E9),E9&lt;0),AND(ISNUMBER(F9),F9&lt;0),AND(ISNUMBER(G9),G9&lt;0),AND(ISNUMBER(H9),H9&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E9),E9&gt;E$4),AND(ISNUMBER(F9),F9&gt;F$4),AND(ISNUMBER(G9),G9&gt;G$4),AND(ISNUMBER(H9),H9&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G9),K9="still failed: presented from the executed notebook",G9&gt;=$G$4),"DEMO RULE",IF(COUNT(E9:H9)+COUNTIF(E9:H9,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E9="","GD ","")&amp;IF(F9="","group part ","")&amp;IF(G9="","presentation and defence ","")&amp;IF(H9="","mock","")),IF(COUNTIF(E9:H9,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E9="ABSENT","GD ","")&amp;IF(F9="ABSENT","group part ","")&amp;IF(G9="ABSENT","presentation and defence ","")&amp;IF(H9="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E9&lt;&gt;"",NOT(ISNUMBER(E9)),E9&lt;&gt;"ABSENT"),AND(F9&lt;&gt;"",NOT(ISNUMBER(F9)),F9&lt;&gt;"ABSENT"),AND(G9&lt;&gt;"",NOT(ISNUMBER(G9)),G9&lt;&gt;"ABSENT"),AND(H9&lt;&gt;"",NOT(ISNUMBER(H9)),H9&lt;&gt;"ABSENT"),AND(F9&lt;&gt;"",NOT(ISNUMBER(F9))),AND(ISNUMBER(E9),E9&lt;0),AND(ISNUMBER(F9),F9&lt;0),AND(ISNUMBER(G9),G9&lt;0),AND(ISNUMBER(H9),H9&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E9),E9&gt;E$4),AND(ISNUMBER(F9),F9&gt;F$4),AND(ISNUMBER(G9),G9&gt;G$4),AND(ISNUMBER(H9),H9&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F9),SUMPRODUCT(($B$6:$B$40=B9)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F9))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G9),K9="still failed: presented from the executed notebook",G9&gt;=$G$4),"DEMO RULE",IF(COUNT(E9:H9)+COUNTIF(E9:H9,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E9="","GD ","")&amp;IF(F9="","group part ","")&amp;IF(G9="","presentation and defence ","")&amp;IF(H9="","mock","")),IF(COUNTIF(E9:H9,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E9="ABSENT","GD ","")&amp;IF(F9="ABSENT","group part ","")&amp;IF(G9="ABSENT","presentation and defence ","")&amp;IF(H9="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M9" s="10" t="n"/>
@@ -1414,7 +1414,7 @@
         <v/>
       </c>
       <c r="L10" s="9">
-        <f>IF(OR(AND(E10&lt;&gt;"",NOT(ISNUMBER(E10)),E10&lt;&gt;"ABSENT"),AND(F10&lt;&gt;"",NOT(ISNUMBER(F10)),F10&lt;&gt;"ABSENT"),AND(G10&lt;&gt;"",NOT(ISNUMBER(G10)),G10&lt;&gt;"ABSENT"),AND(H10&lt;&gt;"",NOT(ISNUMBER(H10)),H10&lt;&gt;"ABSENT"),AND(ISNUMBER(E10),E10&lt;0),AND(ISNUMBER(F10),F10&lt;0),AND(ISNUMBER(G10),G10&lt;0),AND(ISNUMBER(H10),H10&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E10),E10&gt;E$4),AND(ISNUMBER(F10),F10&gt;F$4),AND(ISNUMBER(G10),G10&gt;G$4),AND(ISNUMBER(H10),H10&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G10),K10="still failed: presented from the executed notebook",G10&gt;=$G$4),"DEMO RULE",IF(COUNT(E10:H10)+COUNTIF(E10:H10,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E10="","GD ","")&amp;IF(F10="","group part ","")&amp;IF(G10="","presentation and defence ","")&amp;IF(H10="","mock","")),IF(COUNTIF(E10:H10,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E10="ABSENT","GD ","")&amp;IF(F10="ABSENT","group part ","")&amp;IF(G10="ABSENT","presentation and defence ","")&amp;IF(H10="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E10&lt;&gt;"",NOT(ISNUMBER(E10)),E10&lt;&gt;"ABSENT"),AND(F10&lt;&gt;"",NOT(ISNUMBER(F10)),F10&lt;&gt;"ABSENT"),AND(G10&lt;&gt;"",NOT(ISNUMBER(G10)),G10&lt;&gt;"ABSENT"),AND(H10&lt;&gt;"",NOT(ISNUMBER(H10)),H10&lt;&gt;"ABSENT"),AND(F10&lt;&gt;"",NOT(ISNUMBER(F10))),AND(ISNUMBER(E10),E10&lt;0),AND(ISNUMBER(F10),F10&lt;0),AND(ISNUMBER(G10),G10&lt;0),AND(ISNUMBER(H10),H10&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E10),E10&gt;E$4),AND(ISNUMBER(F10),F10&gt;F$4),AND(ISNUMBER(G10),G10&gt;G$4),AND(ISNUMBER(H10),H10&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F10),SUMPRODUCT(($B$6:$B$40=B10)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F10))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G10),K10="still failed: presented from the executed notebook",G10&gt;=$G$4),"DEMO RULE",IF(COUNT(E10:H10)+COUNTIF(E10:H10,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E10="","GD ","")&amp;IF(F10="","group part ","")&amp;IF(G10="","presentation and defence ","")&amp;IF(H10="","mock","")),IF(COUNTIF(E10:H10,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E10="ABSENT","GD ","")&amp;IF(F10="ABSENT","group part ","")&amp;IF(G10="ABSENT","presentation and defence ","")&amp;IF(H10="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M10" s="10" t="n"/>
@@ -1457,7 +1457,7 @@
         <v/>
       </c>
       <c r="L11" s="9">
-        <f>IF(OR(AND(E11&lt;&gt;"",NOT(ISNUMBER(E11)),E11&lt;&gt;"ABSENT"),AND(F11&lt;&gt;"",NOT(ISNUMBER(F11)),F11&lt;&gt;"ABSENT"),AND(G11&lt;&gt;"",NOT(ISNUMBER(G11)),G11&lt;&gt;"ABSENT"),AND(H11&lt;&gt;"",NOT(ISNUMBER(H11)),H11&lt;&gt;"ABSENT"),AND(ISNUMBER(E11),E11&lt;0),AND(ISNUMBER(F11),F11&lt;0),AND(ISNUMBER(G11),G11&lt;0),AND(ISNUMBER(H11),H11&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E11),E11&gt;E$4),AND(ISNUMBER(F11),F11&gt;F$4),AND(ISNUMBER(G11),G11&gt;G$4),AND(ISNUMBER(H11),H11&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G11),K11="still failed: presented from the executed notebook",G11&gt;=$G$4),"DEMO RULE",IF(COUNT(E11:H11)+COUNTIF(E11:H11,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E11="","GD ","")&amp;IF(F11="","group part ","")&amp;IF(G11="","presentation and defence ","")&amp;IF(H11="","mock","")),IF(COUNTIF(E11:H11,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E11="ABSENT","GD ","")&amp;IF(F11="ABSENT","group part ","")&amp;IF(G11="ABSENT","presentation and defence ","")&amp;IF(H11="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E11&lt;&gt;"",NOT(ISNUMBER(E11)),E11&lt;&gt;"ABSENT"),AND(F11&lt;&gt;"",NOT(ISNUMBER(F11)),F11&lt;&gt;"ABSENT"),AND(G11&lt;&gt;"",NOT(ISNUMBER(G11)),G11&lt;&gt;"ABSENT"),AND(H11&lt;&gt;"",NOT(ISNUMBER(H11)),H11&lt;&gt;"ABSENT"),AND(F11&lt;&gt;"",NOT(ISNUMBER(F11))),AND(ISNUMBER(E11),E11&lt;0),AND(ISNUMBER(F11),F11&lt;0),AND(ISNUMBER(G11),G11&lt;0),AND(ISNUMBER(H11),H11&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E11),E11&gt;E$4),AND(ISNUMBER(F11),F11&gt;F$4),AND(ISNUMBER(G11),G11&gt;G$4),AND(ISNUMBER(H11),H11&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F11),SUMPRODUCT(($B$6:$B$40=B11)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F11))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G11),K11="still failed: presented from the executed notebook",G11&gt;=$G$4),"DEMO RULE",IF(COUNT(E11:H11)+COUNTIF(E11:H11,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E11="","GD ","")&amp;IF(F11="","group part ","")&amp;IF(G11="","presentation and defence ","")&amp;IF(H11="","mock","")),IF(COUNTIF(E11:H11,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E11="ABSENT","GD ","")&amp;IF(F11="ABSENT","group part ","")&amp;IF(G11="ABSENT","presentation and defence ","")&amp;IF(H11="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M11" s="10" t="n"/>
@@ -1500,7 +1500,7 @@
         <v/>
       </c>
       <c r="L12" s="9">
-        <f>IF(OR(AND(E12&lt;&gt;"",NOT(ISNUMBER(E12)),E12&lt;&gt;"ABSENT"),AND(F12&lt;&gt;"",NOT(ISNUMBER(F12)),F12&lt;&gt;"ABSENT"),AND(G12&lt;&gt;"",NOT(ISNUMBER(G12)),G12&lt;&gt;"ABSENT"),AND(H12&lt;&gt;"",NOT(ISNUMBER(H12)),H12&lt;&gt;"ABSENT"),AND(ISNUMBER(E12),E12&lt;0),AND(ISNUMBER(F12),F12&lt;0),AND(ISNUMBER(G12),G12&lt;0),AND(ISNUMBER(H12),H12&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E12),E12&gt;E$4),AND(ISNUMBER(F12),F12&gt;F$4),AND(ISNUMBER(G12),G12&gt;G$4),AND(ISNUMBER(H12),H12&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G12),K12="still failed: presented from the executed notebook",G12&gt;=$G$4),"DEMO RULE",IF(COUNT(E12:H12)+COUNTIF(E12:H12,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E12="","GD ","")&amp;IF(F12="","group part ","")&amp;IF(G12="","presentation and defence ","")&amp;IF(H12="","mock","")),IF(COUNTIF(E12:H12,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E12="ABSENT","GD ","")&amp;IF(F12="ABSENT","group part ","")&amp;IF(G12="ABSENT","presentation and defence ","")&amp;IF(H12="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E12&lt;&gt;"",NOT(ISNUMBER(E12)),E12&lt;&gt;"ABSENT"),AND(F12&lt;&gt;"",NOT(ISNUMBER(F12)),F12&lt;&gt;"ABSENT"),AND(G12&lt;&gt;"",NOT(ISNUMBER(G12)),G12&lt;&gt;"ABSENT"),AND(H12&lt;&gt;"",NOT(ISNUMBER(H12)),H12&lt;&gt;"ABSENT"),AND(F12&lt;&gt;"",NOT(ISNUMBER(F12))),AND(ISNUMBER(E12),E12&lt;0),AND(ISNUMBER(F12),F12&lt;0),AND(ISNUMBER(G12),G12&lt;0),AND(ISNUMBER(H12),H12&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E12),E12&gt;E$4),AND(ISNUMBER(F12),F12&gt;F$4),AND(ISNUMBER(G12),G12&gt;G$4),AND(ISNUMBER(H12),H12&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F12),SUMPRODUCT(($B$6:$B$40=B12)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F12))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G12),K12="still failed: presented from the executed notebook",G12&gt;=$G$4),"DEMO RULE",IF(COUNT(E12:H12)+COUNTIF(E12:H12,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E12="","GD ","")&amp;IF(F12="","group part ","")&amp;IF(G12="","presentation and defence ","")&amp;IF(H12="","mock","")),IF(COUNTIF(E12:H12,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E12="ABSENT","GD ","")&amp;IF(F12="ABSENT","group part ","")&amp;IF(G12="ABSENT","presentation and defence ","")&amp;IF(H12="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M12" s="10" t="n"/>
@@ -1543,7 +1543,7 @@
         <v/>
       </c>
       <c r="L13" s="9">
-        <f>IF(OR(AND(E13&lt;&gt;"",NOT(ISNUMBER(E13)),E13&lt;&gt;"ABSENT"),AND(F13&lt;&gt;"",NOT(ISNUMBER(F13)),F13&lt;&gt;"ABSENT"),AND(G13&lt;&gt;"",NOT(ISNUMBER(G13)),G13&lt;&gt;"ABSENT"),AND(H13&lt;&gt;"",NOT(ISNUMBER(H13)),H13&lt;&gt;"ABSENT"),AND(ISNUMBER(E13),E13&lt;0),AND(ISNUMBER(F13),F13&lt;0),AND(ISNUMBER(G13),G13&lt;0),AND(ISNUMBER(H13),H13&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E13),E13&gt;E$4),AND(ISNUMBER(F13),F13&gt;F$4),AND(ISNUMBER(G13),G13&gt;G$4),AND(ISNUMBER(H13),H13&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G13),K13="still failed: presented from the executed notebook",G13&gt;=$G$4),"DEMO RULE",IF(COUNT(E13:H13)+COUNTIF(E13:H13,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E13="","GD ","")&amp;IF(F13="","group part ","")&amp;IF(G13="","presentation and defence ","")&amp;IF(H13="","mock","")),IF(COUNTIF(E13:H13,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E13="ABSENT","GD ","")&amp;IF(F13="ABSENT","group part ","")&amp;IF(G13="ABSENT","presentation and defence ","")&amp;IF(H13="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E13&lt;&gt;"",NOT(ISNUMBER(E13)),E13&lt;&gt;"ABSENT"),AND(F13&lt;&gt;"",NOT(ISNUMBER(F13)),F13&lt;&gt;"ABSENT"),AND(G13&lt;&gt;"",NOT(ISNUMBER(G13)),G13&lt;&gt;"ABSENT"),AND(H13&lt;&gt;"",NOT(ISNUMBER(H13)),H13&lt;&gt;"ABSENT"),AND(F13&lt;&gt;"",NOT(ISNUMBER(F13))),AND(ISNUMBER(E13),E13&lt;0),AND(ISNUMBER(F13),F13&lt;0),AND(ISNUMBER(G13),G13&lt;0),AND(ISNUMBER(H13),H13&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E13),E13&gt;E$4),AND(ISNUMBER(F13),F13&gt;F$4),AND(ISNUMBER(G13),G13&gt;G$4),AND(ISNUMBER(H13),H13&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F13),SUMPRODUCT(($B$6:$B$40=B13)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F13))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G13),K13="still failed: presented from the executed notebook",G13&gt;=$G$4),"DEMO RULE",IF(COUNT(E13:H13)+COUNTIF(E13:H13,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E13="","GD ","")&amp;IF(F13="","group part ","")&amp;IF(G13="","presentation and defence ","")&amp;IF(H13="","mock","")),IF(COUNTIF(E13:H13,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E13="ABSENT","GD ","")&amp;IF(F13="ABSENT","group part ","")&amp;IF(G13="ABSENT","presentation and defence ","")&amp;IF(H13="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M13" s="10" t="n"/>
@@ -1586,7 +1586,7 @@
         <v/>
       </c>
       <c r="L14" s="9">
-        <f>IF(OR(AND(E14&lt;&gt;"",NOT(ISNUMBER(E14)),E14&lt;&gt;"ABSENT"),AND(F14&lt;&gt;"",NOT(ISNUMBER(F14)),F14&lt;&gt;"ABSENT"),AND(G14&lt;&gt;"",NOT(ISNUMBER(G14)),G14&lt;&gt;"ABSENT"),AND(H14&lt;&gt;"",NOT(ISNUMBER(H14)),H14&lt;&gt;"ABSENT"),AND(ISNUMBER(E14),E14&lt;0),AND(ISNUMBER(F14),F14&lt;0),AND(ISNUMBER(G14),G14&lt;0),AND(ISNUMBER(H14),H14&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E14),E14&gt;E$4),AND(ISNUMBER(F14),F14&gt;F$4),AND(ISNUMBER(G14),G14&gt;G$4),AND(ISNUMBER(H14),H14&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G14),K14="still failed: presented from the executed notebook",G14&gt;=$G$4),"DEMO RULE",IF(COUNT(E14:H14)+COUNTIF(E14:H14,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E14="","GD ","")&amp;IF(F14="","group part ","")&amp;IF(G14="","presentation and defence ","")&amp;IF(H14="","mock","")),IF(COUNTIF(E14:H14,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E14="ABSENT","GD ","")&amp;IF(F14="ABSENT","group part ","")&amp;IF(G14="ABSENT","presentation and defence ","")&amp;IF(H14="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E14&lt;&gt;"",NOT(ISNUMBER(E14)),E14&lt;&gt;"ABSENT"),AND(F14&lt;&gt;"",NOT(ISNUMBER(F14)),F14&lt;&gt;"ABSENT"),AND(G14&lt;&gt;"",NOT(ISNUMBER(G14)),G14&lt;&gt;"ABSENT"),AND(H14&lt;&gt;"",NOT(ISNUMBER(H14)),H14&lt;&gt;"ABSENT"),AND(F14&lt;&gt;"",NOT(ISNUMBER(F14))),AND(ISNUMBER(E14),E14&lt;0),AND(ISNUMBER(F14),F14&lt;0),AND(ISNUMBER(G14),G14&lt;0),AND(ISNUMBER(H14),H14&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E14),E14&gt;E$4),AND(ISNUMBER(F14),F14&gt;F$4),AND(ISNUMBER(G14),G14&gt;G$4),AND(ISNUMBER(H14),H14&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F14),SUMPRODUCT(($B$6:$B$40=B14)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F14))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G14),K14="still failed: presented from the executed notebook",G14&gt;=$G$4),"DEMO RULE",IF(COUNT(E14:H14)+COUNTIF(E14:H14,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E14="","GD ","")&amp;IF(F14="","group part ","")&amp;IF(G14="","presentation and defence ","")&amp;IF(H14="","mock","")),IF(COUNTIF(E14:H14,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E14="ABSENT","GD ","")&amp;IF(F14="ABSENT","group part ","")&amp;IF(G14="ABSENT","presentation and defence ","")&amp;IF(H14="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M14" s="10" t="n"/>
@@ -1629,7 +1629,7 @@
         <v/>
       </c>
       <c r="L15" s="9">
-        <f>IF(OR(AND(E15&lt;&gt;"",NOT(ISNUMBER(E15)),E15&lt;&gt;"ABSENT"),AND(F15&lt;&gt;"",NOT(ISNUMBER(F15)),F15&lt;&gt;"ABSENT"),AND(G15&lt;&gt;"",NOT(ISNUMBER(G15)),G15&lt;&gt;"ABSENT"),AND(H15&lt;&gt;"",NOT(ISNUMBER(H15)),H15&lt;&gt;"ABSENT"),AND(ISNUMBER(E15),E15&lt;0),AND(ISNUMBER(F15),F15&lt;0),AND(ISNUMBER(G15),G15&lt;0),AND(ISNUMBER(H15),H15&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E15),E15&gt;E$4),AND(ISNUMBER(F15),F15&gt;F$4),AND(ISNUMBER(G15),G15&gt;G$4),AND(ISNUMBER(H15),H15&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G15),K15="still failed: presented from the executed notebook",G15&gt;=$G$4),"DEMO RULE",IF(COUNT(E15:H15)+COUNTIF(E15:H15,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E15="","GD ","")&amp;IF(F15="","group part ","")&amp;IF(G15="","presentation and defence ","")&amp;IF(H15="","mock","")),IF(COUNTIF(E15:H15,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E15="ABSENT","GD ","")&amp;IF(F15="ABSENT","group part ","")&amp;IF(G15="ABSENT","presentation and defence ","")&amp;IF(H15="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E15&lt;&gt;"",NOT(ISNUMBER(E15)),E15&lt;&gt;"ABSENT"),AND(F15&lt;&gt;"",NOT(ISNUMBER(F15)),F15&lt;&gt;"ABSENT"),AND(G15&lt;&gt;"",NOT(ISNUMBER(G15)),G15&lt;&gt;"ABSENT"),AND(H15&lt;&gt;"",NOT(ISNUMBER(H15)),H15&lt;&gt;"ABSENT"),AND(F15&lt;&gt;"",NOT(ISNUMBER(F15))),AND(ISNUMBER(E15),E15&lt;0),AND(ISNUMBER(F15),F15&lt;0),AND(ISNUMBER(G15),G15&lt;0),AND(ISNUMBER(H15),H15&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E15),E15&gt;E$4),AND(ISNUMBER(F15),F15&gt;F$4),AND(ISNUMBER(G15),G15&gt;G$4),AND(ISNUMBER(H15),H15&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F15),SUMPRODUCT(($B$6:$B$40=B15)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F15))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G15),K15="still failed: presented from the executed notebook",G15&gt;=$G$4),"DEMO RULE",IF(COUNT(E15:H15)+COUNTIF(E15:H15,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E15="","GD ","")&amp;IF(F15="","group part ","")&amp;IF(G15="","presentation and defence ","")&amp;IF(H15="","mock","")),IF(COUNTIF(E15:H15,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E15="ABSENT","GD ","")&amp;IF(F15="ABSENT","group part ","")&amp;IF(G15="ABSENT","presentation and defence ","")&amp;IF(H15="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M15" s="10" t="n"/>
@@ -1672,7 +1672,7 @@
         <v/>
       </c>
       <c r="L16" s="9">
-        <f>IF(OR(AND(E16&lt;&gt;"",NOT(ISNUMBER(E16)),E16&lt;&gt;"ABSENT"),AND(F16&lt;&gt;"",NOT(ISNUMBER(F16)),F16&lt;&gt;"ABSENT"),AND(G16&lt;&gt;"",NOT(ISNUMBER(G16)),G16&lt;&gt;"ABSENT"),AND(H16&lt;&gt;"",NOT(ISNUMBER(H16)),H16&lt;&gt;"ABSENT"),AND(ISNUMBER(E16),E16&lt;0),AND(ISNUMBER(F16),F16&lt;0),AND(ISNUMBER(G16),G16&lt;0),AND(ISNUMBER(H16),H16&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E16),E16&gt;E$4),AND(ISNUMBER(F16),F16&gt;F$4),AND(ISNUMBER(G16),G16&gt;G$4),AND(ISNUMBER(H16),H16&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G16),K16="still failed: presented from the executed notebook",G16&gt;=$G$4),"DEMO RULE",IF(COUNT(E16:H16)+COUNTIF(E16:H16,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E16="","GD ","")&amp;IF(F16="","group part ","")&amp;IF(G16="","presentation and defence ","")&amp;IF(H16="","mock","")),IF(COUNTIF(E16:H16,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E16="ABSENT","GD ","")&amp;IF(F16="ABSENT","group part ","")&amp;IF(G16="ABSENT","presentation and defence ","")&amp;IF(H16="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E16&lt;&gt;"",NOT(ISNUMBER(E16)),E16&lt;&gt;"ABSENT"),AND(F16&lt;&gt;"",NOT(ISNUMBER(F16)),F16&lt;&gt;"ABSENT"),AND(G16&lt;&gt;"",NOT(ISNUMBER(G16)),G16&lt;&gt;"ABSENT"),AND(H16&lt;&gt;"",NOT(ISNUMBER(H16)),H16&lt;&gt;"ABSENT"),AND(F16&lt;&gt;"",NOT(ISNUMBER(F16))),AND(ISNUMBER(E16),E16&lt;0),AND(ISNUMBER(F16),F16&lt;0),AND(ISNUMBER(G16),G16&lt;0),AND(ISNUMBER(H16),H16&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E16),E16&gt;E$4),AND(ISNUMBER(F16),F16&gt;F$4),AND(ISNUMBER(G16),G16&gt;G$4),AND(ISNUMBER(H16),H16&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F16),SUMPRODUCT(($B$6:$B$40=B16)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F16))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G16),K16="still failed: presented from the executed notebook",G16&gt;=$G$4),"DEMO RULE",IF(COUNT(E16:H16)+COUNTIF(E16:H16,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E16="","GD ","")&amp;IF(F16="","group part ","")&amp;IF(G16="","presentation and defence ","")&amp;IF(H16="","mock","")),IF(COUNTIF(E16:H16,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E16="ABSENT","GD ","")&amp;IF(F16="ABSENT","group part ","")&amp;IF(G16="ABSENT","presentation and defence ","")&amp;IF(H16="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M16" s="10" t="n"/>
@@ -1715,7 +1715,7 @@
         <v/>
       </c>
       <c r="L17" s="9">
-        <f>IF(OR(AND(E17&lt;&gt;"",NOT(ISNUMBER(E17)),E17&lt;&gt;"ABSENT"),AND(F17&lt;&gt;"",NOT(ISNUMBER(F17)),F17&lt;&gt;"ABSENT"),AND(G17&lt;&gt;"",NOT(ISNUMBER(G17)),G17&lt;&gt;"ABSENT"),AND(H17&lt;&gt;"",NOT(ISNUMBER(H17)),H17&lt;&gt;"ABSENT"),AND(ISNUMBER(E17),E17&lt;0),AND(ISNUMBER(F17),F17&lt;0),AND(ISNUMBER(G17),G17&lt;0),AND(ISNUMBER(H17),H17&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E17),E17&gt;E$4),AND(ISNUMBER(F17),F17&gt;F$4),AND(ISNUMBER(G17),G17&gt;G$4),AND(ISNUMBER(H17),H17&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G17),K17="still failed: presented from the executed notebook",G17&gt;=$G$4),"DEMO RULE",IF(COUNT(E17:H17)+COUNTIF(E17:H17,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E17="","GD ","")&amp;IF(F17="","group part ","")&amp;IF(G17="","presentation and defence ","")&amp;IF(H17="","mock","")),IF(COUNTIF(E17:H17,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E17="ABSENT","GD ","")&amp;IF(F17="ABSENT","group part ","")&amp;IF(G17="ABSENT","presentation and defence ","")&amp;IF(H17="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E17&lt;&gt;"",NOT(ISNUMBER(E17)),E17&lt;&gt;"ABSENT"),AND(F17&lt;&gt;"",NOT(ISNUMBER(F17)),F17&lt;&gt;"ABSENT"),AND(G17&lt;&gt;"",NOT(ISNUMBER(G17)),G17&lt;&gt;"ABSENT"),AND(H17&lt;&gt;"",NOT(ISNUMBER(H17)),H17&lt;&gt;"ABSENT"),AND(F17&lt;&gt;"",NOT(ISNUMBER(F17))),AND(ISNUMBER(E17),E17&lt;0),AND(ISNUMBER(F17),F17&lt;0),AND(ISNUMBER(G17),G17&lt;0),AND(ISNUMBER(H17),H17&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E17),E17&gt;E$4),AND(ISNUMBER(F17),F17&gt;F$4),AND(ISNUMBER(G17),G17&gt;G$4),AND(ISNUMBER(H17),H17&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F17),SUMPRODUCT(($B$6:$B$40=B17)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F17))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G17),K17="still failed: presented from the executed notebook",G17&gt;=$G$4),"DEMO RULE",IF(COUNT(E17:H17)+COUNTIF(E17:H17,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E17="","GD ","")&amp;IF(F17="","group part ","")&amp;IF(G17="","presentation and defence ","")&amp;IF(H17="","mock","")),IF(COUNTIF(E17:H17,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E17="ABSENT","GD ","")&amp;IF(F17="ABSENT","group part ","")&amp;IF(G17="ABSENT","presentation and defence ","")&amp;IF(H17="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M17" s="10" t="n"/>
@@ -1758,7 +1758,7 @@
         <v/>
       </c>
       <c r="L18" s="9">
-        <f>IF(OR(AND(E18&lt;&gt;"",NOT(ISNUMBER(E18)),E18&lt;&gt;"ABSENT"),AND(F18&lt;&gt;"",NOT(ISNUMBER(F18)),F18&lt;&gt;"ABSENT"),AND(G18&lt;&gt;"",NOT(ISNUMBER(G18)),G18&lt;&gt;"ABSENT"),AND(H18&lt;&gt;"",NOT(ISNUMBER(H18)),H18&lt;&gt;"ABSENT"),AND(ISNUMBER(E18),E18&lt;0),AND(ISNUMBER(F18),F18&lt;0),AND(ISNUMBER(G18),G18&lt;0),AND(ISNUMBER(H18),H18&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E18),E18&gt;E$4),AND(ISNUMBER(F18),F18&gt;F$4),AND(ISNUMBER(G18),G18&gt;G$4),AND(ISNUMBER(H18),H18&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G18),K18="still failed: presented from the executed notebook",G18&gt;=$G$4),"DEMO RULE",IF(COUNT(E18:H18)+COUNTIF(E18:H18,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E18="","GD ","")&amp;IF(F18="","group part ","")&amp;IF(G18="","presentation and defence ","")&amp;IF(H18="","mock","")),IF(COUNTIF(E18:H18,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E18="ABSENT","GD ","")&amp;IF(F18="ABSENT","group part ","")&amp;IF(G18="ABSENT","presentation and defence ","")&amp;IF(H18="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E18&lt;&gt;"",NOT(ISNUMBER(E18)),E18&lt;&gt;"ABSENT"),AND(F18&lt;&gt;"",NOT(ISNUMBER(F18)),F18&lt;&gt;"ABSENT"),AND(G18&lt;&gt;"",NOT(ISNUMBER(G18)),G18&lt;&gt;"ABSENT"),AND(H18&lt;&gt;"",NOT(ISNUMBER(H18)),H18&lt;&gt;"ABSENT"),AND(F18&lt;&gt;"",NOT(ISNUMBER(F18))),AND(ISNUMBER(E18),E18&lt;0),AND(ISNUMBER(F18),F18&lt;0),AND(ISNUMBER(G18),G18&lt;0),AND(ISNUMBER(H18),H18&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E18),E18&gt;E$4),AND(ISNUMBER(F18),F18&gt;F$4),AND(ISNUMBER(G18),G18&gt;G$4),AND(ISNUMBER(H18),H18&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F18),SUMPRODUCT(($B$6:$B$40=B18)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F18))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G18),K18="still failed: presented from the executed notebook",G18&gt;=$G$4),"DEMO RULE",IF(COUNT(E18:H18)+COUNTIF(E18:H18,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E18="","GD ","")&amp;IF(F18="","group part ","")&amp;IF(G18="","presentation and defence ","")&amp;IF(H18="","mock","")),IF(COUNTIF(E18:H18,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E18="ABSENT","GD ","")&amp;IF(F18="ABSENT","group part ","")&amp;IF(G18="ABSENT","presentation and defence ","")&amp;IF(H18="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M18" s="10" t="n"/>
@@ -1801,7 +1801,7 @@
         <v/>
       </c>
       <c r="L19" s="9">
-        <f>IF(OR(AND(E19&lt;&gt;"",NOT(ISNUMBER(E19)),E19&lt;&gt;"ABSENT"),AND(F19&lt;&gt;"",NOT(ISNUMBER(F19)),F19&lt;&gt;"ABSENT"),AND(G19&lt;&gt;"",NOT(ISNUMBER(G19)),G19&lt;&gt;"ABSENT"),AND(H19&lt;&gt;"",NOT(ISNUMBER(H19)),H19&lt;&gt;"ABSENT"),AND(ISNUMBER(E19),E19&lt;0),AND(ISNUMBER(F19),F19&lt;0),AND(ISNUMBER(G19),G19&lt;0),AND(ISNUMBER(H19),H19&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E19),E19&gt;E$4),AND(ISNUMBER(F19),F19&gt;F$4),AND(ISNUMBER(G19),G19&gt;G$4),AND(ISNUMBER(H19),H19&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G19),K19="still failed: presented from the executed notebook",G19&gt;=$G$4),"DEMO RULE",IF(COUNT(E19:H19)+COUNTIF(E19:H19,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E19="","GD ","")&amp;IF(F19="","group part ","")&amp;IF(G19="","presentation and defence ","")&amp;IF(H19="","mock","")),IF(COUNTIF(E19:H19,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E19="ABSENT","GD ","")&amp;IF(F19="ABSENT","group part ","")&amp;IF(G19="ABSENT","presentation and defence ","")&amp;IF(H19="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E19&lt;&gt;"",NOT(ISNUMBER(E19)),E19&lt;&gt;"ABSENT"),AND(F19&lt;&gt;"",NOT(ISNUMBER(F19)),F19&lt;&gt;"ABSENT"),AND(G19&lt;&gt;"",NOT(ISNUMBER(G19)),G19&lt;&gt;"ABSENT"),AND(H19&lt;&gt;"",NOT(ISNUMBER(H19)),H19&lt;&gt;"ABSENT"),AND(F19&lt;&gt;"",NOT(ISNUMBER(F19))),AND(ISNUMBER(E19),E19&lt;0),AND(ISNUMBER(F19),F19&lt;0),AND(ISNUMBER(G19),G19&lt;0),AND(ISNUMBER(H19),H19&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E19),E19&gt;E$4),AND(ISNUMBER(F19),F19&gt;F$4),AND(ISNUMBER(G19),G19&gt;G$4),AND(ISNUMBER(H19),H19&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F19),SUMPRODUCT(($B$6:$B$40=B19)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F19))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G19),K19="still failed: presented from the executed notebook",G19&gt;=$G$4),"DEMO RULE",IF(COUNT(E19:H19)+COUNTIF(E19:H19,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E19="","GD ","")&amp;IF(F19="","group part ","")&amp;IF(G19="","presentation and defence ","")&amp;IF(H19="","mock","")),IF(COUNTIF(E19:H19,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E19="ABSENT","GD ","")&amp;IF(F19="ABSENT","group part ","")&amp;IF(G19="ABSENT","presentation and defence ","")&amp;IF(H19="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M19" s="10" t="n"/>
@@ -1844,7 +1844,7 @@
         <v/>
       </c>
       <c r="L20" s="9">
-        <f>IF(OR(AND(E20&lt;&gt;"",NOT(ISNUMBER(E20)),E20&lt;&gt;"ABSENT"),AND(F20&lt;&gt;"",NOT(ISNUMBER(F20)),F20&lt;&gt;"ABSENT"),AND(G20&lt;&gt;"",NOT(ISNUMBER(G20)),G20&lt;&gt;"ABSENT"),AND(H20&lt;&gt;"",NOT(ISNUMBER(H20)),H20&lt;&gt;"ABSENT"),AND(ISNUMBER(E20),E20&lt;0),AND(ISNUMBER(F20),F20&lt;0),AND(ISNUMBER(G20),G20&lt;0),AND(ISNUMBER(H20),H20&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E20),E20&gt;E$4),AND(ISNUMBER(F20),F20&gt;F$4),AND(ISNUMBER(G20),G20&gt;G$4),AND(ISNUMBER(H20),H20&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G20),K20="still failed: presented from the executed notebook",G20&gt;=$G$4),"DEMO RULE",IF(COUNT(E20:H20)+COUNTIF(E20:H20,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E20="","GD ","")&amp;IF(F20="","group part ","")&amp;IF(G20="","presentation and defence ","")&amp;IF(H20="","mock","")),IF(COUNTIF(E20:H20,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E20="ABSENT","GD ","")&amp;IF(F20="ABSENT","group part ","")&amp;IF(G20="ABSENT","presentation and defence ","")&amp;IF(H20="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E20&lt;&gt;"",NOT(ISNUMBER(E20)),E20&lt;&gt;"ABSENT"),AND(F20&lt;&gt;"",NOT(ISNUMBER(F20)),F20&lt;&gt;"ABSENT"),AND(G20&lt;&gt;"",NOT(ISNUMBER(G20)),G20&lt;&gt;"ABSENT"),AND(H20&lt;&gt;"",NOT(ISNUMBER(H20)),H20&lt;&gt;"ABSENT"),AND(F20&lt;&gt;"",NOT(ISNUMBER(F20))),AND(ISNUMBER(E20),E20&lt;0),AND(ISNUMBER(F20),F20&lt;0),AND(ISNUMBER(G20),G20&lt;0),AND(ISNUMBER(H20),H20&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E20),E20&gt;E$4),AND(ISNUMBER(F20),F20&gt;F$4),AND(ISNUMBER(G20),G20&gt;G$4),AND(ISNUMBER(H20),H20&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F20),SUMPRODUCT(($B$6:$B$40=B20)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F20))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G20),K20="still failed: presented from the executed notebook",G20&gt;=$G$4),"DEMO RULE",IF(COUNT(E20:H20)+COUNTIF(E20:H20,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E20="","GD ","")&amp;IF(F20="","group part ","")&amp;IF(G20="","presentation and defence ","")&amp;IF(H20="","mock","")),IF(COUNTIF(E20:H20,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E20="ABSENT","GD ","")&amp;IF(F20="ABSENT","group part ","")&amp;IF(G20="ABSENT","presentation and defence ","")&amp;IF(H20="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M20" s="10" t="n"/>
@@ -1887,7 +1887,7 @@
         <v/>
       </c>
       <c r="L21" s="9">
-        <f>IF(OR(AND(E21&lt;&gt;"",NOT(ISNUMBER(E21)),E21&lt;&gt;"ABSENT"),AND(F21&lt;&gt;"",NOT(ISNUMBER(F21)),F21&lt;&gt;"ABSENT"),AND(G21&lt;&gt;"",NOT(ISNUMBER(G21)),G21&lt;&gt;"ABSENT"),AND(H21&lt;&gt;"",NOT(ISNUMBER(H21)),H21&lt;&gt;"ABSENT"),AND(ISNUMBER(E21),E21&lt;0),AND(ISNUMBER(F21),F21&lt;0),AND(ISNUMBER(G21),G21&lt;0),AND(ISNUMBER(H21),H21&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E21),E21&gt;E$4),AND(ISNUMBER(F21),F21&gt;F$4),AND(ISNUMBER(G21),G21&gt;G$4),AND(ISNUMBER(H21),H21&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G21),K21="still failed: presented from the executed notebook",G21&gt;=$G$4),"DEMO RULE",IF(COUNT(E21:H21)+COUNTIF(E21:H21,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E21="","GD ","")&amp;IF(F21="","group part ","")&amp;IF(G21="","presentation and defence ","")&amp;IF(H21="","mock","")),IF(COUNTIF(E21:H21,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E21="ABSENT","GD ","")&amp;IF(F21="ABSENT","group part ","")&amp;IF(G21="ABSENT","presentation and defence ","")&amp;IF(H21="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E21&lt;&gt;"",NOT(ISNUMBER(E21)),E21&lt;&gt;"ABSENT"),AND(F21&lt;&gt;"",NOT(ISNUMBER(F21)),F21&lt;&gt;"ABSENT"),AND(G21&lt;&gt;"",NOT(ISNUMBER(G21)),G21&lt;&gt;"ABSENT"),AND(H21&lt;&gt;"",NOT(ISNUMBER(H21)),H21&lt;&gt;"ABSENT"),AND(F21&lt;&gt;"",NOT(ISNUMBER(F21))),AND(ISNUMBER(E21),E21&lt;0),AND(ISNUMBER(F21),F21&lt;0),AND(ISNUMBER(G21),G21&lt;0),AND(ISNUMBER(H21),H21&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E21),E21&gt;E$4),AND(ISNUMBER(F21),F21&gt;F$4),AND(ISNUMBER(G21),G21&gt;G$4),AND(ISNUMBER(H21),H21&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F21),SUMPRODUCT(($B$6:$B$40=B21)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F21))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G21),K21="still failed: presented from the executed notebook",G21&gt;=$G$4),"DEMO RULE",IF(COUNT(E21:H21)+COUNTIF(E21:H21,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E21="","GD ","")&amp;IF(F21="","group part ","")&amp;IF(G21="","presentation and defence ","")&amp;IF(H21="","mock","")),IF(COUNTIF(E21:H21,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E21="ABSENT","GD ","")&amp;IF(F21="ABSENT","group part ","")&amp;IF(G21="ABSENT","presentation and defence ","")&amp;IF(H21="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M21" s="10" t="n"/>
@@ -1930,7 +1930,7 @@
         <v/>
       </c>
       <c r="L22" s="9">
-        <f>IF(OR(AND(E22&lt;&gt;"",NOT(ISNUMBER(E22)),E22&lt;&gt;"ABSENT"),AND(F22&lt;&gt;"",NOT(ISNUMBER(F22)),F22&lt;&gt;"ABSENT"),AND(G22&lt;&gt;"",NOT(ISNUMBER(G22)),G22&lt;&gt;"ABSENT"),AND(H22&lt;&gt;"",NOT(ISNUMBER(H22)),H22&lt;&gt;"ABSENT"),AND(ISNUMBER(E22),E22&lt;0),AND(ISNUMBER(F22),F22&lt;0),AND(ISNUMBER(G22),G22&lt;0),AND(ISNUMBER(H22),H22&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E22),E22&gt;E$4),AND(ISNUMBER(F22),F22&gt;F$4),AND(ISNUMBER(G22),G22&gt;G$4),AND(ISNUMBER(H22),H22&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G22),K22="still failed: presented from the executed notebook",G22&gt;=$G$4),"DEMO RULE",IF(COUNT(E22:H22)+COUNTIF(E22:H22,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E22="","GD ","")&amp;IF(F22="","group part ","")&amp;IF(G22="","presentation and defence ","")&amp;IF(H22="","mock","")),IF(COUNTIF(E22:H22,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E22="ABSENT","GD ","")&amp;IF(F22="ABSENT","group part ","")&amp;IF(G22="ABSENT","presentation and defence ","")&amp;IF(H22="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E22&lt;&gt;"",NOT(ISNUMBER(E22)),E22&lt;&gt;"ABSENT"),AND(F22&lt;&gt;"",NOT(ISNUMBER(F22)),F22&lt;&gt;"ABSENT"),AND(G22&lt;&gt;"",NOT(ISNUMBER(G22)),G22&lt;&gt;"ABSENT"),AND(H22&lt;&gt;"",NOT(ISNUMBER(H22)),H22&lt;&gt;"ABSENT"),AND(F22&lt;&gt;"",NOT(ISNUMBER(F22))),AND(ISNUMBER(E22),E22&lt;0),AND(ISNUMBER(F22),F22&lt;0),AND(ISNUMBER(G22),G22&lt;0),AND(ISNUMBER(H22),H22&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E22),E22&gt;E$4),AND(ISNUMBER(F22),F22&gt;F$4),AND(ISNUMBER(G22),G22&gt;G$4),AND(ISNUMBER(H22),H22&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F22),SUMPRODUCT(($B$6:$B$40=B22)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F22))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G22),K22="still failed: presented from the executed notebook",G22&gt;=$G$4),"DEMO RULE",IF(COUNT(E22:H22)+COUNTIF(E22:H22,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E22="","GD ","")&amp;IF(F22="","group part ","")&amp;IF(G22="","presentation and defence ","")&amp;IF(H22="","mock","")),IF(COUNTIF(E22:H22,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E22="ABSENT","GD ","")&amp;IF(F22="ABSENT","group part ","")&amp;IF(G22="ABSENT","presentation and defence ","")&amp;IF(H22="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M22" s="10" t="n"/>
@@ -1973,7 +1973,7 @@
         <v/>
       </c>
       <c r="L23" s="9">
-        <f>IF(OR(AND(E23&lt;&gt;"",NOT(ISNUMBER(E23)),E23&lt;&gt;"ABSENT"),AND(F23&lt;&gt;"",NOT(ISNUMBER(F23)),F23&lt;&gt;"ABSENT"),AND(G23&lt;&gt;"",NOT(ISNUMBER(G23)),G23&lt;&gt;"ABSENT"),AND(H23&lt;&gt;"",NOT(ISNUMBER(H23)),H23&lt;&gt;"ABSENT"),AND(ISNUMBER(E23),E23&lt;0),AND(ISNUMBER(F23),F23&lt;0),AND(ISNUMBER(G23),G23&lt;0),AND(ISNUMBER(H23),H23&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E23),E23&gt;E$4),AND(ISNUMBER(F23),F23&gt;F$4),AND(ISNUMBER(G23),G23&gt;G$4),AND(ISNUMBER(H23),H23&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G23),K23="still failed: presented from the executed notebook",G23&gt;=$G$4),"DEMO RULE",IF(COUNT(E23:H23)+COUNTIF(E23:H23,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E23="","GD ","")&amp;IF(F23="","group part ","")&amp;IF(G23="","presentation and defence ","")&amp;IF(H23="","mock","")),IF(COUNTIF(E23:H23,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E23="ABSENT","GD ","")&amp;IF(F23="ABSENT","group part ","")&amp;IF(G23="ABSENT","presentation and defence ","")&amp;IF(H23="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E23&lt;&gt;"",NOT(ISNUMBER(E23)),E23&lt;&gt;"ABSENT"),AND(F23&lt;&gt;"",NOT(ISNUMBER(F23)),F23&lt;&gt;"ABSENT"),AND(G23&lt;&gt;"",NOT(ISNUMBER(G23)),G23&lt;&gt;"ABSENT"),AND(H23&lt;&gt;"",NOT(ISNUMBER(H23)),H23&lt;&gt;"ABSENT"),AND(F23&lt;&gt;"",NOT(ISNUMBER(F23))),AND(ISNUMBER(E23),E23&lt;0),AND(ISNUMBER(F23),F23&lt;0),AND(ISNUMBER(G23),G23&lt;0),AND(ISNUMBER(H23),H23&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E23),E23&gt;E$4),AND(ISNUMBER(F23),F23&gt;F$4),AND(ISNUMBER(G23),G23&gt;G$4),AND(ISNUMBER(H23),H23&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F23),SUMPRODUCT(($B$6:$B$40=B23)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F23))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G23),K23="still failed: presented from the executed notebook",G23&gt;=$G$4),"DEMO RULE",IF(COUNT(E23:H23)+COUNTIF(E23:H23,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E23="","GD ","")&amp;IF(F23="","group part ","")&amp;IF(G23="","presentation and defence ","")&amp;IF(H23="","mock","")),IF(COUNTIF(E23:H23,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E23="ABSENT","GD ","")&amp;IF(F23="ABSENT","group part ","")&amp;IF(G23="ABSENT","presentation and defence ","")&amp;IF(H23="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M23" s="10" t="n"/>
@@ -2016,7 +2016,7 @@
         <v/>
       </c>
       <c r="L24" s="9">
-        <f>IF(OR(AND(E24&lt;&gt;"",NOT(ISNUMBER(E24)),E24&lt;&gt;"ABSENT"),AND(F24&lt;&gt;"",NOT(ISNUMBER(F24)),F24&lt;&gt;"ABSENT"),AND(G24&lt;&gt;"",NOT(ISNUMBER(G24)),G24&lt;&gt;"ABSENT"),AND(H24&lt;&gt;"",NOT(ISNUMBER(H24)),H24&lt;&gt;"ABSENT"),AND(ISNUMBER(E24),E24&lt;0),AND(ISNUMBER(F24),F24&lt;0),AND(ISNUMBER(G24),G24&lt;0),AND(ISNUMBER(H24),H24&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E24),E24&gt;E$4),AND(ISNUMBER(F24),F24&gt;F$4),AND(ISNUMBER(G24),G24&gt;G$4),AND(ISNUMBER(H24),H24&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G24),K24="still failed: presented from the executed notebook",G24&gt;=$G$4),"DEMO RULE",IF(COUNT(E24:H24)+COUNTIF(E24:H24,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E24="","GD ","")&amp;IF(F24="","group part ","")&amp;IF(G24="","presentation and defence ","")&amp;IF(H24="","mock","")),IF(COUNTIF(E24:H24,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E24="ABSENT","GD ","")&amp;IF(F24="ABSENT","group part ","")&amp;IF(G24="ABSENT","presentation and defence ","")&amp;IF(H24="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E24&lt;&gt;"",NOT(ISNUMBER(E24)),E24&lt;&gt;"ABSENT"),AND(F24&lt;&gt;"",NOT(ISNUMBER(F24)),F24&lt;&gt;"ABSENT"),AND(G24&lt;&gt;"",NOT(ISNUMBER(G24)),G24&lt;&gt;"ABSENT"),AND(H24&lt;&gt;"",NOT(ISNUMBER(H24)),H24&lt;&gt;"ABSENT"),AND(F24&lt;&gt;"",NOT(ISNUMBER(F24))),AND(ISNUMBER(E24),E24&lt;0),AND(ISNUMBER(F24),F24&lt;0),AND(ISNUMBER(G24),G24&lt;0),AND(ISNUMBER(H24),H24&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E24),E24&gt;E$4),AND(ISNUMBER(F24),F24&gt;F$4),AND(ISNUMBER(G24),G24&gt;G$4),AND(ISNUMBER(H24),H24&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F24),SUMPRODUCT(($B$6:$B$40=B24)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F24))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G24),K24="still failed: presented from the executed notebook",G24&gt;=$G$4),"DEMO RULE",IF(COUNT(E24:H24)+COUNTIF(E24:H24,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E24="","GD ","")&amp;IF(F24="","group part ","")&amp;IF(G24="","presentation and defence ","")&amp;IF(H24="","mock","")),IF(COUNTIF(E24:H24,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E24="ABSENT","GD ","")&amp;IF(F24="ABSENT","group part ","")&amp;IF(G24="ABSENT","presentation and defence ","")&amp;IF(H24="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M24" s="10" t="n"/>
@@ -2059,7 +2059,7 @@
         <v/>
       </c>
       <c r="L25" s="9">
-        <f>IF(OR(AND(E25&lt;&gt;"",NOT(ISNUMBER(E25)),E25&lt;&gt;"ABSENT"),AND(F25&lt;&gt;"",NOT(ISNUMBER(F25)),F25&lt;&gt;"ABSENT"),AND(G25&lt;&gt;"",NOT(ISNUMBER(G25)),G25&lt;&gt;"ABSENT"),AND(H25&lt;&gt;"",NOT(ISNUMBER(H25)),H25&lt;&gt;"ABSENT"),AND(ISNUMBER(E25),E25&lt;0),AND(ISNUMBER(F25),F25&lt;0),AND(ISNUMBER(G25),G25&lt;0),AND(ISNUMBER(H25),H25&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E25),E25&gt;E$4),AND(ISNUMBER(F25),F25&gt;F$4),AND(ISNUMBER(G25),G25&gt;G$4),AND(ISNUMBER(H25),H25&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G25),K25="still failed: presented from the executed notebook",G25&gt;=$G$4),"DEMO RULE",IF(COUNT(E25:H25)+COUNTIF(E25:H25,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E25="","GD ","")&amp;IF(F25="","group part ","")&amp;IF(G25="","presentation and defence ","")&amp;IF(H25="","mock","")),IF(COUNTIF(E25:H25,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E25="ABSENT","GD ","")&amp;IF(F25="ABSENT","group part ","")&amp;IF(G25="ABSENT","presentation and defence ","")&amp;IF(H25="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E25&lt;&gt;"",NOT(ISNUMBER(E25)),E25&lt;&gt;"ABSENT"),AND(F25&lt;&gt;"",NOT(ISNUMBER(F25)),F25&lt;&gt;"ABSENT"),AND(G25&lt;&gt;"",NOT(ISNUMBER(G25)),G25&lt;&gt;"ABSENT"),AND(H25&lt;&gt;"",NOT(ISNUMBER(H25)),H25&lt;&gt;"ABSENT"),AND(F25&lt;&gt;"",NOT(ISNUMBER(F25))),AND(ISNUMBER(E25),E25&lt;0),AND(ISNUMBER(F25),F25&lt;0),AND(ISNUMBER(G25),G25&lt;0),AND(ISNUMBER(H25),H25&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E25),E25&gt;E$4),AND(ISNUMBER(F25),F25&gt;F$4),AND(ISNUMBER(G25),G25&gt;G$4),AND(ISNUMBER(H25),H25&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F25),SUMPRODUCT(($B$6:$B$40=B25)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F25))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G25),K25="still failed: presented from the executed notebook",G25&gt;=$G$4),"DEMO RULE",IF(COUNT(E25:H25)+COUNTIF(E25:H25,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E25="","GD ","")&amp;IF(F25="","group part ","")&amp;IF(G25="","presentation and defence ","")&amp;IF(H25="","mock","")),IF(COUNTIF(E25:H25,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E25="ABSENT","GD ","")&amp;IF(F25="ABSENT","group part ","")&amp;IF(G25="ABSENT","presentation and defence ","")&amp;IF(H25="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M25" s="10" t="n"/>
@@ -2102,7 +2102,7 @@
         <v/>
       </c>
       <c r="L26" s="9">
-        <f>IF(OR(AND(E26&lt;&gt;"",NOT(ISNUMBER(E26)),E26&lt;&gt;"ABSENT"),AND(F26&lt;&gt;"",NOT(ISNUMBER(F26)),F26&lt;&gt;"ABSENT"),AND(G26&lt;&gt;"",NOT(ISNUMBER(G26)),G26&lt;&gt;"ABSENT"),AND(H26&lt;&gt;"",NOT(ISNUMBER(H26)),H26&lt;&gt;"ABSENT"),AND(ISNUMBER(E26),E26&lt;0),AND(ISNUMBER(F26),F26&lt;0),AND(ISNUMBER(G26),G26&lt;0),AND(ISNUMBER(H26),H26&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E26),E26&gt;E$4),AND(ISNUMBER(F26),F26&gt;F$4),AND(ISNUMBER(G26),G26&gt;G$4),AND(ISNUMBER(H26),H26&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G26),K26="still failed: presented from the executed notebook",G26&gt;=$G$4),"DEMO RULE",IF(COUNT(E26:H26)+COUNTIF(E26:H26,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E26="","GD ","")&amp;IF(F26="","group part ","")&amp;IF(G26="","presentation and defence ","")&amp;IF(H26="","mock","")),IF(COUNTIF(E26:H26,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E26="ABSENT","GD ","")&amp;IF(F26="ABSENT","group part ","")&amp;IF(G26="ABSENT","presentation and defence ","")&amp;IF(H26="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E26&lt;&gt;"",NOT(ISNUMBER(E26)),E26&lt;&gt;"ABSENT"),AND(F26&lt;&gt;"",NOT(ISNUMBER(F26)),F26&lt;&gt;"ABSENT"),AND(G26&lt;&gt;"",NOT(ISNUMBER(G26)),G26&lt;&gt;"ABSENT"),AND(H26&lt;&gt;"",NOT(ISNUMBER(H26)),H26&lt;&gt;"ABSENT"),AND(F26&lt;&gt;"",NOT(ISNUMBER(F26))),AND(ISNUMBER(E26),E26&lt;0),AND(ISNUMBER(F26),F26&lt;0),AND(ISNUMBER(G26),G26&lt;0),AND(ISNUMBER(H26),H26&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E26),E26&gt;E$4),AND(ISNUMBER(F26),F26&gt;F$4),AND(ISNUMBER(G26),G26&gt;G$4),AND(ISNUMBER(H26),H26&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F26),SUMPRODUCT(($B$6:$B$40=B26)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F26))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G26),K26="still failed: presented from the executed notebook",G26&gt;=$G$4),"DEMO RULE",IF(COUNT(E26:H26)+COUNTIF(E26:H26,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E26="","GD ","")&amp;IF(F26="","group part ","")&amp;IF(G26="","presentation and defence ","")&amp;IF(H26="","mock","")),IF(COUNTIF(E26:H26,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E26="ABSENT","GD ","")&amp;IF(F26="ABSENT","group part ","")&amp;IF(G26="ABSENT","presentation and defence ","")&amp;IF(H26="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M26" s="10" t="n"/>
@@ -2145,7 +2145,7 @@
         <v/>
       </c>
       <c r="L27" s="9">
-        <f>IF(OR(AND(E27&lt;&gt;"",NOT(ISNUMBER(E27)),E27&lt;&gt;"ABSENT"),AND(F27&lt;&gt;"",NOT(ISNUMBER(F27)),F27&lt;&gt;"ABSENT"),AND(G27&lt;&gt;"",NOT(ISNUMBER(G27)),G27&lt;&gt;"ABSENT"),AND(H27&lt;&gt;"",NOT(ISNUMBER(H27)),H27&lt;&gt;"ABSENT"),AND(ISNUMBER(E27),E27&lt;0),AND(ISNUMBER(F27),F27&lt;0),AND(ISNUMBER(G27),G27&lt;0),AND(ISNUMBER(H27),H27&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E27),E27&gt;E$4),AND(ISNUMBER(F27),F27&gt;F$4),AND(ISNUMBER(G27),G27&gt;G$4),AND(ISNUMBER(H27),H27&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G27),K27="still failed: presented from the executed notebook",G27&gt;=$G$4),"DEMO RULE",IF(COUNT(E27:H27)+COUNTIF(E27:H27,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E27="","GD ","")&amp;IF(F27="","group part ","")&amp;IF(G27="","presentation and defence ","")&amp;IF(H27="","mock","")),IF(COUNTIF(E27:H27,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E27="ABSENT","GD ","")&amp;IF(F27="ABSENT","group part ","")&amp;IF(G27="ABSENT","presentation and defence ","")&amp;IF(H27="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E27&lt;&gt;"",NOT(ISNUMBER(E27)),E27&lt;&gt;"ABSENT"),AND(F27&lt;&gt;"",NOT(ISNUMBER(F27)),F27&lt;&gt;"ABSENT"),AND(G27&lt;&gt;"",NOT(ISNUMBER(G27)),G27&lt;&gt;"ABSENT"),AND(H27&lt;&gt;"",NOT(ISNUMBER(H27)),H27&lt;&gt;"ABSENT"),AND(F27&lt;&gt;"",NOT(ISNUMBER(F27))),AND(ISNUMBER(E27),E27&lt;0),AND(ISNUMBER(F27),F27&lt;0),AND(ISNUMBER(G27),G27&lt;0),AND(ISNUMBER(H27),H27&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E27),E27&gt;E$4),AND(ISNUMBER(F27),F27&gt;F$4),AND(ISNUMBER(G27),G27&gt;G$4),AND(ISNUMBER(H27),H27&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F27),SUMPRODUCT(($B$6:$B$40=B27)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F27))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G27),K27="still failed: presented from the executed notebook",G27&gt;=$G$4),"DEMO RULE",IF(COUNT(E27:H27)+COUNTIF(E27:H27,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E27="","GD ","")&amp;IF(F27="","group part ","")&amp;IF(G27="","presentation and defence ","")&amp;IF(H27="","mock","")),IF(COUNTIF(E27:H27,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E27="ABSENT","GD ","")&amp;IF(F27="ABSENT","group part ","")&amp;IF(G27="ABSENT","presentation and defence ","")&amp;IF(H27="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M27" s="10" t="n"/>
@@ -2188,7 +2188,7 @@
         <v/>
       </c>
       <c r="L28" s="9">
-        <f>IF(OR(AND(E28&lt;&gt;"",NOT(ISNUMBER(E28)),E28&lt;&gt;"ABSENT"),AND(F28&lt;&gt;"",NOT(ISNUMBER(F28)),F28&lt;&gt;"ABSENT"),AND(G28&lt;&gt;"",NOT(ISNUMBER(G28)),G28&lt;&gt;"ABSENT"),AND(H28&lt;&gt;"",NOT(ISNUMBER(H28)),H28&lt;&gt;"ABSENT"),AND(ISNUMBER(E28),E28&lt;0),AND(ISNUMBER(F28),F28&lt;0),AND(ISNUMBER(G28),G28&lt;0),AND(ISNUMBER(H28),H28&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E28),E28&gt;E$4),AND(ISNUMBER(F28),F28&gt;F$4),AND(ISNUMBER(G28),G28&gt;G$4),AND(ISNUMBER(H28),H28&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G28),K28="still failed: presented from the executed notebook",G28&gt;=$G$4),"DEMO RULE",IF(COUNT(E28:H28)+COUNTIF(E28:H28,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E28="","GD ","")&amp;IF(F28="","group part ","")&amp;IF(G28="","presentation and defence ","")&amp;IF(H28="","mock","")),IF(COUNTIF(E28:H28,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E28="ABSENT","GD ","")&amp;IF(F28="ABSENT","group part ","")&amp;IF(G28="ABSENT","presentation and defence ","")&amp;IF(H28="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E28&lt;&gt;"",NOT(ISNUMBER(E28)),E28&lt;&gt;"ABSENT"),AND(F28&lt;&gt;"",NOT(ISNUMBER(F28)),F28&lt;&gt;"ABSENT"),AND(G28&lt;&gt;"",NOT(ISNUMBER(G28)),G28&lt;&gt;"ABSENT"),AND(H28&lt;&gt;"",NOT(ISNUMBER(H28)),H28&lt;&gt;"ABSENT"),AND(F28&lt;&gt;"",NOT(ISNUMBER(F28))),AND(ISNUMBER(E28),E28&lt;0),AND(ISNUMBER(F28),F28&lt;0),AND(ISNUMBER(G28),G28&lt;0),AND(ISNUMBER(H28),H28&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E28),E28&gt;E$4),AND(ISNUMBER(F28),F28&gt;F$4),AND(ISNUMBER(G28),G28&gt;G$4),AND(ISNUMBER(H28),H28&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F28),SUMPRODUCT(($B$6:$B$40=B28)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F28))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G28),K28="still failed: presented from the executed notebook",G28&gt;=$G$4),"DEMO RULE",IF(COUNT(E28:H28)+COUNTIF(E28:H28,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E28="","GD ","")&amp;IF(F28="","group part ","")&amp;IF(G28="","presentation and defence ","")&amp;IF(H28="","mock","")),IF(COUNTIF(E28:H28,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E28="ABSENT","GD ","")&amp;IF(F28="ABSENT","group part ","")&amp;IF(G28="ABSENT","presentation and defence ","")&amp;IF(H28="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M28" s="10" t="n"/>
@@ -2231,7 +2231,7 @@
         <v/>
       </c>
       <c r="L29" s="9">
-        <f>IF(OR(AND(E29&lt;&gt;"",NOT(ISNUMBER(E29)),E29&lt;&gt;"ABSENT"),AND(F29&lt;&gt;"",NOT(ISNUMBER(F29)),F29&lt;&gt;"ABSENT"),AND(G29&lt;&gt;"",NOT(ISNUMBER(G29)),G29&lt;&gt;"ABSENT"),AND(H29&lt;&gt;"",NOT(ISNUMBER(H29)),H29&lt;&gt;"ABSENT"),AND(ISNUMBER(E29),E29&lt;0),AND(ISNUMBER(F29),F29&lt;0),AND(ISNUMBER(G29),G29&lt;0),AND(ISNUMBER(H29),H29&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E29),E29&gt;E$4),AND(ISNUMBER(F29),F29&gt;F$4),AND(ISNUMBER(G29),G29&gt;G$4),AND(ISNUMBER(H29),H29&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G29),K29="still failed: presented from the executed notebook",G29&gt;=$G$4),"DEMO RULE",IF(COUNT(E29:H29)+COUNTIF(E29:H29,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E29="","GD ","")&amp;IF(F29="","group part ","")&amp;IF(G29="","presentation and defence ","")&amp;IF(H29="","mock","")),IF(COUNTIF(E29:H29,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E29="ABSENT","GD ","")&amp;IF(F29="ABSENT","group part ","")&amp;IF(G29="ABSENT","presentation and defence ","")&amp;IF(H29="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E29&lt;&gt;"",NOT(ISNUMBER(E29)),E29&lt;&gt;"ABSENT"),AND(F29&lt;&gt;"",NOT(ISNUMBER(F29)),F29&lt;&gt;"ABSENT"),AND(G29&lt;&gt;"",NOT(ISNUMBER(G29)),G29&lt;&gt;"ABSENT"),AND(H29&lt;&gt;"",NOT(ISNUMBER(H29)),H29&lt;&gt;"ABSENT"),AND(F29&lt;&gt;"",NOT(ISNUMBER(F29))),AND(ISNUMBER(E29),E29&lt;0),AND(ISNUMBER(F29),F29&lt;0),AND(ISNUMBER(G29),G29&lt;0),AND(ISNUMBER(H29),H29&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E29),E29&gt;E$4),AND(ISNUMBER(F29),F29&gt;F$4),AND(ISNUMBER(G29),G29&gt;G$4),AND(ISNUMBER(H29),H29&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F29),SUMPRODUCT(($B$6:$B$40=B29)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F29))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G29),K29="still failed: presented from the executed notebook",G29&gt;=$G$4),"DEMO RULE",IF(COUNT(E29:H29)+COUNTIF(E29:H29,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E29="","GD ","")&amp;IF(F29="","group part ","")&amp;IF(G29="","presentation and defence ","")&amp;IF(H29="","mock","")),IF(COUNTIF(E29:H29,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E29="ABSENT","GD ","")&amp;IF(F29="ABSENT","group part ","")&amp;IF(G29="ABSENT","presentation and defence ","")&amp;IF(H29="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M29" s="10" t="n"/>
@@ -2274,7 +2274,7 @@
         <v/>
       </c>
       <c r="L30" s="9">
-        <f>IF(OR(AND(E30&lt;&gt;"",NOT(ISNUMBER(E30)),E30&lt;&gt;"ABSENT"),AND(F30&lt;&gt;"",NOT(ISNUMBER(F30)),F30&lt;&gt;"ABSENT"),AND(G30&lt;&gt;"",NOT(ISNUMBER(G30)),G30&lt;&gt;"ABSENT"),AND(H30&lt;&gt;"",NOT(ISNUMBER(H30)),H30&lt;&gt;"ABSENT"),AND(ISNUMBER(E30),E30&lt;0),AND(ISNUMBER(F30),F30&lt;0),AND(ISNUMBER(G30),G30&lt;0),AND(ISNUMBER(H30),H30&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E30),E30&gt;E$4),AND(ISNUMBER(F30),F30&gt;F$4),AND(ISNUMBER(G30),G30&gt;G$4),AND(ISNUMBER(H30),H30&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G30),K30="still failed: presented from the executed notebook",G30&gt;=$G$4),"DEMO RULE",IF(COUNT(E30:H30)+COUNTIF(E30:H30,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E30="","GD ","")&amp;IF(F30="","group part ","")&amp;IF(G30="","presentation and defence ","")&amp;IF(H30="","mock","")),IF(COUNTIF(E30:H30,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E30="ABSENT","GD ","")&amp;IF(F30="ABSENT","group part ","")&amp;IF(G30="ABSENT","presentation and defence ","")&amp;IF(H30="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E30&lt;&gt;"",NOT(ISNUMBER(E30)),E30&lt;&gt;"ABSENT"),AND(F30&lt;&gt;"",NOT(ISNUMBER(F30)),F30&lt;&gt;"ABSENT"),AND(G30&lt;&gt;"",NOT(ISNUMBER(G30)),G30&lt;&gt;"ABSENT"),AND(H30&lt;&gt;"",NOT(ISNUMBER(H30)),H30&lt;&gt;"ABSENT"),AND(F30&lt;&gt;"",NOT(ISNUMBER(F30))),AND(ISNUMBER(E30),E30&lt;0),AND(ISNUMBER(F30),F30&lt;0),AND(ISNUMBER(G30),G30&lt;0),AND(ISNUMBER(H30),H30&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E30),E30&gt;E$4),AND(ISNUMBER(F30),F30&gt;F$4),AND(ISNUMBER(G30),G30&gt;G$4),AND(ISNUMBER(H30),H30&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F30),SUMPRODUCT(($B$6:$B$40=B30)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F30))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G30),K30="still failed: presented from the executed notebook",G30&gt;=$G$4),"DEMO RULE",IF(COUNT(E30:H30)+COUNTIF(E30:H30,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E30="","GD ","")&amp;IF(F30="","group part ","")&amp;IF(G30="","presentation and defence ","")&amp;IF(H30="","mock","")),IF(COUNTIF(E30:H30,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E30="ABSENT","GD ","")&amp;IF(F30="ABSENT","group part ","")&amp;IF(G30="ABSENT","presentation and defence ","")&amp;IF(H30="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M30" s="10" t="n"/>
@@ -2317,7 +2317,7 @@
         <v/>
       </c>
       <c r="L31" s="9">
-        <f>IF(OR(AND(E31&lt;&gt;"",NOT(ISNUMBER(E31)),E31&lt;&gt;"ABSENT"),AND(F31&lt;&gt;"",NOT(ISNUMBER(F31)),F31&lt;&gt;"ABSENT"),AND(G31&lt;&gt;"",NOT(ISNUMBER(G31)),G31&lt;&gt;"ABSENT"),AND(H31&lt;&gt;"",NOT(ISNUMBER(H31)),H31&lt;&gt;"ABSENT"),AND(ISNUMBER(E31),E31&lt;0),AND(ISNUMBER(F31),F31&lt;0),AND(ISNUMBER(G31),G31&lt;0),AND(ISNUMBER(H31),H31&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E31),E31&gt;E$4),AND(ISNUMBER(F31),F31&gt;F$4),AND(ISNUMBER(G31),G31&gt;G$4),AND(ISNUMBER(H31),H31&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G31),K31="still failed: presented from the executed notebook",G31&gt;=$G$4),"DEMO RULE",IF(COUNT(E31:H31)+COUNTIF(E31:H31,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E31="","GD ","")&amp;IF(F31="","group part ","")&amp;IF(G31="","presentation and defence ","")&amp;IF(H31="","mock","")),IF(COUNTIF(E31:H31,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E31="ABSENT","GD ","")&amp;IF(F31="ABSENT","group part ","")&amp;IF(G31="ABSENT","presentation and defence ","")&amp;IF(H31="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E31&lt;&gt;"",NOT(ISNUMBER(E31)),E31&lt;&gt;"ABSENT"),AND(F31&lt;&gt;"",NOT(ISNUMBER(F31)),F31&lt;&gt;"ABSENT"),AND(G31&lt;&gt;"",NOT(ISNUMBER(G31)),G31&lt;&gt;"ABSENT"),AND(H31&lt;&gt;"",NOT(ISNUMBER(H31)),H31&lt;&gt;"ABSENT"),AND(F31&lt;&gt;"",NOT(ISNUMBER(F31))),AND(ISNUMBER(E31),E31&lt;0),AND(ISNUMBER(F31),F31&lt;0),AND(ISNUMBER(G31),G31&lt;0),AND(ISNUMBER(H31),H31&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E31),E31&gt;E$4),AND(ISNUMBER(F31),F31&gt;F$4),AND(ISNUMBER(G31),G31&gt;G$4),AND(ISNUMBER(H31),H31&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F31),SUMPRODUCT(($B$6:$B$40=B31)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F31))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G31),K31="still failed: presented from the executed notebook",G31&gt;=$G$4),"DEMO RULE",IF(COUNT(E31:H31)+COUNTIF(E31:H31,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E31="","GD ","")&amp;IF(F31="","group part ","")&amp;IF(G31="","presentation and defence ","")&amp;IF(H31="","mock","")),IF(COUNTIF(E31:H31,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E31="ABSENT","GD ","")&amp;IF(F31="ABSENT","group part ","")&amp;IF(G31="ABSENT","presentation and defence ","")&amp;IF(H31="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M31" s="10" t="n"/>
@@ -2360,7 +2360,7 @@
         <v/>
       </c>
       <c r="L32" s="9">
-        <f>IF(OR(AND(E32&lt;&gt;"",NOT(ISNUMBER(E32)),E32&lt;&gt;"ABSENT"),AND(F32&lt;&gt;"",NOT(ISNUMBER(F32)),F32&lt;&gt;"ABSENT"),AND(G32&lt;&gt;"",NOT(ISNUMBER(G32)),G32&lt;&gt;"ABSENT"),AND(H32&lt;&gt;"",NOT(ISNUMBER(H32)),H32&lt;&gt;"ABSENT"),AND(ISNUMBER(E32),E32&lt;0),AND(ISNUMBER(F32),F32&lt;0),AND(ISNUMBER(G32),G32&lt;0),AND(ISNUMBER(H32),H32&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E32),E32&gt;E$4),AND(ISNUMBER(F32),F32&gt;F$4),AND(ISNUMBER(G32),G32&gt;G$4),AND(ISNUMBER(H32),H32&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G32),K32="still failed: presented from the executed notebook",G32&gt;=$G$4),"DEMO RULE",IF(COUNT(E32:H32)+COUNTIF(E32:H32,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E32="","GD ","")&amp;IF(F32="","group part ","")&amp;IF(G32="","presentation and defence ","")&amp;IF(H32="","mock","")),IF(COUNTIF(E32:H32,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E32="ABSENT","GD ","")&amp;IF(F32="ABSENT","group part ","")&amp;IF(G32="ABSENT","presentation and defence ","")&amp;IF(H32="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E32&lt;&gt;"",NOT(ISNUMBER(E32)),E32&lt;&gt;"ABSENT"),AND(F32&lt;&gt;"",NOT(ISNUMBER(F32)),F32&lt;&gt;"ABSENT"),AND(G32&lt;&gt;"",NOT(ISNUMBER(G32)),G32&lt;&gt;"ABSENT"),AND(H32&lt;&gt;"",NOT(ISNUMBER(H32)),H32&lt;&gt;"ABSENT"),AND(F32&lt;&gt;"",NOT(ISNUMBER(F32))),AND(ISNUMBER(E32),E32&lt;0),AND(ISNUMBER(F32),F32&lt;0),AND(ISNUMBER(G32),G32&lt;0),AND(ISNUMBER(H32),H32&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E32),E32&gt;E$4),AND(ISNUMBER(F32),F32&gt;F$4),AND(ISNUMBER(G32),G32&gt;G$4),AND(ISNUMBER(H32),H32&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F32),SUMPRODUCT(($B$6:$B$40=B32)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F32))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G32),K32="still failed: presented from the executed notebook",G32&gt;=$G$4),"DEMO RULE",IF(COUNT(E32:H32)+COUNTIF(E32:H32,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E32="","GD ","")&amp;IF(F32="","group part ","")&amp;IF(G32="","presentation and defence ","")&amp;IF(H32="","mock","")),IF(COUNTIF(E32:H32,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E32="ABSENT","GD ","")&amp;IF(F32="ABSENT","group part ","")&amp;IF(G32="ABSENT","presentation and defence ","")&amp;IF(H32="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M32" s="10" t="n"/>
@@ -2403,7 +2403,7 @@
         <v/>
       </c>
       <c r="L33" s="9">
-        <f>IF(OR(AND(E33&lt;&gt;"",NOT(ISNUMBER(E33)),E33&lt;&gt;"ABSENT"),AND(F33&lt;&gt;"",NOT(ISNUMBER(F33)),F33&lt;&gt;"ABSENT"),AND(G33&lt;&gt;"",NOT(ISNUMBER(G33)),G33&lt;&gt;"ABSENT"),AND(H33&lt;&gt;"",NOT(ISNUMBER(H33)),H33&lt;&gt;"ABSENT"),AND(ISNUMBER(E33),E33&lt;0),AND(ISNUMBER(F33),F33&lt;0),AND(ISNUMBER(G33),G33&lt;0),AND(ISNUMBER(H33),H33&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E33),E33&gt;E$4),AND(ISNUMBER(F33),F33&gt;F$4),AND(ISNUMBER(G33),G33&gt;G$4),AND(ISNUMBER(H33),H33&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G33),K33="still failed: presented from the executed notebook",G33&gt;=$G$4),"DEMO RULE",IF(COUNT(E33:H33)+COUNTIF(E33:H33,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E33="","GD ","")&amp;IF(F33="","group part ","")&amp;IF(G33="","presentation and defence ","")&amp;IF(H33="","mock","")),IF(COUNTIF(E33:H33,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E33="ABSENT","GD ","")&amp;IF(F33="ABSENT","group part ","")&amp;IF(G33="ABSENT","presentation and defence ","")&amp;IF(H33="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E33&lt;&gt;"",NOT(ISNUMBER(E33)),E33&lt;&gt;"ABSENT"),AND(F33&lt;&gt;"",NOT(ISNUMBER(F33)),F33&lt;&gt;"ABSENT"),AND(G33&lt;&gt;"",NOT(ISNUMBER(G33)),G33&lt;&gt;"ABSENT"),AND(H33&lt;&gt;"",NOT(ISNUMBER(H33)),H33&lt;&gt;"ABSENT"),AND(F33&lt;&gt;"",NOT(ISNUMBER(F33))),AND(ISNUMBER(E33),E33&lt;0),AND(ISNUMBER(F33),F33&lt;0),AND(ISNUMBER(G33),G33&lt;0),AND(ISNUMBER(H33),H33&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E33),E33&gt;E$4),AND(ISNUMBER(F33),F33&gt;F$4),AND(ISNUMBER(G33),G33&gt;G$4),AND(ISNUMBER(H33),H33&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F33),SUMPRODUCT(($B$6:$B$40=B33)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F33))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G33),K33="still failed: presented from the executed notebook",G33&gt;=$G$4),"DEMO RULE",IF(COUNT(E33:H33)+COUNTIF(E33:H33,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E33="","GD ","")&amp;IF(F33="","group part ","")&amp;IF(G33="","presentation and defence ","")&amp;IF(H33="","mock","")),IF(COUNTIF(E33:H33,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E33="ABSENT","GD ","")&amp;IF(F33="ABSENT","group part ","")&amp;IF(G33="ABSENT","presentation and defence ","")&amp;IF(H33="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M33" s="10" t="n"/>
@@ -2446,7 +2446,7 @@
         <v/>
       </c>
       <c r="L34" s="9">
-        <f>IF(OR(AND(E34&lt;&gt;"",NOT(ISNUMBER(E34)),E34&lt;&gt;"ABSENT"),AND(F34&lt;&gt;"",NOT(ISNUMBER(F34)),F34&lt;&gt;"ABSENT"),AND(G34&lt;&gt;"",NOT(ISNUMBER(G34)),G34&lt;&gt;"ABSENT"),AND(H34&lt;&gt;"",NOT(ISNUMBER(H34)),H34&lt;&gt;"ABSENT"),AND(ISNUMBER(E34),E34&lt;0),AND(ISNUMBER(F34),F34&lt;0),AND(ISNUMBER(G34),G34&lt;0),AND(ISNUMBER(H34),H34&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E34),E34&gt;E$4),AND(ISNUMBER(F34),F34&gt;F$4),AND(ISNUMBER(G34),G34&gt;G$4),AND(ISNUMBER(H34),H34&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G34),K34="still failed: presented from the executed notebook",G34&gt;=$G$4),"DEMO RULE",IF(COUNT(E34:H34)+COUNTIF(E34:H34,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E34="","GD ","")&amp;IF(F34="","group part ","")&amp;IF(G34="","presentation and defence ","")&amp;IF(H34="","mock","")),IF(COUNTIF(E34:H34,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E34="ABSENT","GD ","")&amp;IF(F34="ABSENT","group part ","")&amp;IF(G34="ABSENT","presentation and defence ","")&amp;IF(H34="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E34&lt;&gt;"",NOT(ISNUMBER(E34)),E34&lt;&gt;"ABSENT"),AND(F34&lt;&gt;"",NOT(ISNUMBER(F34)),F34&lt;&gt;"ABSENT"),AND(G34&lt;&gt;"",NOT(ISNUMBER(G34)),G34&lt;&gt;"ABSENT"),AND(H34&lt;&gt;"",NOT(ISNUMBER(H34)),H34&lt;&gt;"ABSENT"),AND(F34&lt;&gt;"",NOT(ISNUMBER(F34))),AND(ISNUMBER(E34),E34&lt;0),AND(ISNUMBER(F34),F34&lt;0),AND(ISNUMBER(G34),G34&lt;0),AND(ISNUMBER(H34),H34&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E34),E34&gt;E$4),AND(ISNUMBER(F34),F34&gt;F$4),AND(ISNUMBER(G34),G34&gt;G$4),AND(ISNUMBER(H34),H34&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F34),SUMPRODUCT(($B$6:$B$40=B34)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F34))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G34),K34="still failed: presented from the executed notebook",G34&gt;=$G$4),"DEMO RULE",IF(COUNT(E34:H34)+COUNTIF(E34:H34,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E34="","GD ","")&amp;IF(F34="","group part ","")&amp;IF(G34="","presentation and defence ","")&amp;IF(H34="","mock","")),IF(COUNTIF(E34:H34,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E34="ABSENT","GD ","")&amp;IF(F34="ABSENT","group part ","")&amp;IF(G34="ABSENT","presentation and defence ","")&amp;IF(H34="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M34" s="10" t="n"/>
@@ -2489,7 +2489,7 @@
         <v/>
       </c>
       <c r="L35" s="9">
-        <f>IF(OR(AND(E35&lt;&gt;"",NOT(ISNUMBER(E35)),E35&lt;&gt;"ABSENT"),AND(F35&lt;&gt;"",NOT(ISNUMBER(F35)),F35&lt;&gt;"ABSENT"),AND(G35&lt;&gt;"",NOT(ISNUMBER(G35)),G35&lt;&gt;"ABSENT"),AND(H35&lt;&gt;"",NOT(ISNUMBER(H35)),H35&lt;&gt;"ABSENT"),AND(ISNUMBER(E35),E35&lt;0),AND(ISNUMBER(F35),F35&lt;0),AND(ISNUMBER(G35),G35&lt;0),AND(ISNUMBER(H35),H35&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E35),E35&gt;E$4),AND(ISNUMBER(F35),F35&gt;F$4),AND(ISNUMBER(G35),G35&gt;G$4),AND(ISNUMBER(H35),H35&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G35),K35="still failed: presented from the executed notebook",G35&gt;=$G$4),"DEMO RULE",IF(COUNT(E35:H35)+COUNTIF(E35:H35,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E35="","GD ","")&amp;IF(F35="","group part ","")&amp;IF(G35="","presentation and defence ","")&amp;IF(H35="","mock","")),IF(COUNTIF(E35:H35,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E35="ABSENT","GD ","")&amp;IF(F35="ABSENT","group part ","")&amp;IF(G35="ABSENT","presentation and defence ","")&amp;IF(H35="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E35&lt;&gt;"",NOT(ISNUMBER(E35)),E35&lt;&gt;"ABSENT"),AND(F35&lt;&gt;"",NOT(ISNUMBER(F35)),F35&lt;&gt;"ABSENT"),AND(G35&lt;&gt;"",NOT(ISNUMBER(G35)),G35&lt;&gt;"ABSENT"),AND(H35&lt;&gt;"",NOT(ISNUMBER(H35)),H35&lt;&gt;"ABSENT"),AND(F35&lt;&gt;"",NOT(ISNUMBER(F35))),AND(ISNUMBER(E35),E35&lt;0),AND(ISNUMBER(F35),F35&lt;0),AND(ISNUMBER(G35),G35&lt;0),AND(ISNUMBER(H35),H35&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E35),E35&gt;E$4),AND(ISNUMBER(F35),F35&gt;F$4),AND(ISNUMBER(G35),G35&gt;G$4),AND(ISNUMBER(H35),H35&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F35),SUMPRODUCT(($B$6:$B$40=B35)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F35))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G35),K35="still failed: presented from the executed notebook",G35&gt;=$G$4),"DEMO RULE",IF(COUNT(E35:H35)+COUNTIF(E35:H35,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E35="","GD ","")&amp;IF(F35="","group part ","")&amp;IF(G35="","presentation and defence ","")&amp;IF(H35="","mock","")),IF(COUNTIF(E35:H35,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E35="ABSENT","GD ","")&amp;IF(F35="ABSENT","group part ","")&amp;IF(G35="ABSENT","presentation and defence ","")&amp;IF(H35="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M35" s="10" t="n"/>
@@ -2532,7 +2532,7 @@
         <v/>
       </c>
       <c r="L36" s="9">
-        <f>IF(OR(AND(E36&lt;&gt;"",NOT(ISNUMBER(E36)),E36&lt;&gt;"ABSENT"),AND(F36&lt;&gt;"",NOT(ISNUMBER(F36)),F36&lt;&gt;"ABSENT"),AND(G36&lt;&gt;"",NOT(ISNUMBER(G36)),G36&lt;&gt;"ABSENT"),AND(H36&lt;&gt;"",NOT(ISNUMBER(H36)),H36&lt;&gt;"ABSENT"),AND(ISNUMBER(E36),E36&lt;0),AND(ISNUMBER(F36),F36&lt;0),AND(ISNUMBER(G36),G36&lt;0),AND(ISNUMBER(H36),H36&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E36),E36&gt;E$4),AND(ISNUMBER(F36),F36&gt;F$4),AND(ISNUMBER(G36),G36&gt;G$4),AND(ISNUMBER(H36),H36&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G36),K36="still failed: presented from the executed notebook",G36&gt;=$G$4),"DEMO RULE",IF(COUNT(E36:H36)+COUNTIF(E36:H36,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E36="","GD ","")&amp;IF(F36="","group part ","")&amp;IF(G36="","presentation and defence ","")&amp;IF(H36="","mock","")),IF(COUNTIF(E36:H36,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E36="ABSENT","GD ","")&amp;IF(F36="ABSENT","group part ","")&amp;IF(G36="ABSENT","presentation and defence ","")&amp;IF(H36="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E36&lt;&gt;"",NOT(ISNUMBER(E36)),E36&lt;&gt;"ABSENT"),AND(F36&lt;&gt;"",NOT(ISNUMBER(F36)),F36&lt;&gt;"ABSENT"),AND(G36&lt;&gt;"",NOT(ISNUMBER(G36)),G36&lt;&gt;"ABSENT"),AND(H36&lt;&gt;"",NOT(ISNUMBER(H36)),H36&lt;&gt;"ABSENT"),AND(F36&lt;&gt;"",NOT(ISNUMBER(F36))),AND(ISNUMBER(E36),E36&lt;0),AND(ISNUMBER(F36),F36&lt;0),AND(ISNUMBER(G36),G36&lt;0),AND(ISNUMBER(H36),H36&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E36),E36&gt;E$4),AND(ISNUMBER(F36),F36&gt;F$4),AND(ISNUMBER(G36),G36&gt;G$4),AND(ISNUMBER(H36),H36&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F36),SUMPRODUCT(($B$6:$B$40=B36)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F36))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G36),K36="still failed: presented from the executed notebook",G36&gt;=$G$4),"DEMO RULE",IF(COUNT(E36:H36)+COUNTIF(E36:H36,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E36="","GD ","")&amp;IF(F36="","group part ","")&amp;IF(G36="","presentation and defence ","")&amp;IF(H36="","mock","")),IF(COUNTIF(E36:H36,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E36="ABSENT","GD ","")&amp;IF(F36="ABSENT","group part ","")&amp;IF(G36="ABSENT","presentation and defence ","")&amp;IF(H36="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M36" s="10" t="n"/>
@@ -2575,7 +2575,7 @@
         <v/>
       </c>
       <c r="L37" s="9">
-        <f>IF(OR(AND(E37&lt;&gt;"",NOT(ISNUMBER(E37)),E37&lt;&gt;"ABSENT"),AND(F37&lt;&gt;"",NOT(ISNUMBER(F37)),F37&lt;&gt;"ABSENT"),AND(G37&lt;&gt;"",NOT(ISNUMBER(G37)),G37&lt;&gt;"ABSENT"),AND(H37&lt;&gt;"",NOT(ISNUMBER(H37)),H37&lt;&gt;"ABSENT"),AND(ISNUMBER(E37),E37&lt;0),AND(ISNUMBER(F37),F37&lt;0),AND(ISNUMBER(G37),G37&lt;0),AND(ISNUMBER(H37),H37&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E37),E37&gt;E$4),AND(ISNUMBER(F37),F37&gt;F$4),AND(ISNUMBER(G37),G37&gt;G$4),AND(ISNUMBER(H37),H37&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G37),K37="still failed: presented from the executed notebook",G37&gt;=$G$4),"DEMO RULE",IF(COUNT(E37:H37)+COUNTIF(E37:H37,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E37="","GD ","")&amp;IF(F37="","group part ","")&amp;IF(G37="","presentation and defence ","")&amp;IF(H37="","mock","")),IF(COUNTIF(E37:H37,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E37="ABSENT","GD ","")&amp;IF(F37="ABSENT","group part ","")&amp;IF(G37="ABSENT","presentation and defence ","")&amp;IF(H37="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E37&lt;&gt;"",NOT(ISNUMBER(E37)),E37&lt;&gt;"ABSENT"),AND(F37&lt;&gt;"",NOT(ISNUMBER(F37)),F37&lt;&gt;"ABSENT"),AND(G37&lt;&gt;"",NOT(ISNUMBER(G37)),G37&lt;&gt;"ABSENT"),AND(H37&lt;&gt;"",NOT(ISNUMBER(H37)),H37&lt;&gt;"ABSENT"),AND(F37&lt;&gt;"",NOT(ISNUMBER(F37))),AND(ISNUMBER(E37),E37&lt;0),AND(ISNUMBER(F37),F37&lt;0),AND(ISNUMBER(G37),G37&lt;0),AND(ISNUMBER(H37),H37&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E37),E37&gt;E$4),AND(ISNUMBER(F37),F37&gt;F$4),AND(ISNUMBER(G37),G37&gt;G$4),AND(ISNUMBER(H37),H37&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F37),SUMPRODUCT(($B$6:$B$40=B37)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F37))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G37),K37="still failed: presented from the executed notebook",G37&gt;=$G$4),"DEMO RULE",IF(COUNT(E37:H37)+COUNTIF(E37:H37,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E37="","GD ","")&amp;IF(F37="","group part ","")&amp;IF(G37="","presentation and defence ","")&amp;IF(H37="","mock","")),IF(COUNTIF(E37:H37,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E37="ABSENT","GD ","")&amp;IF(F37="ABSENT","group part ","")&amp;IF(G37="ABSENT","presentation and defence ","")&amp;IF(H37="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M37" s="10" t="n"/>
@@ -2618,7 +2618,7 @@
         <v/>
       </c>
       <c r="L38" s="9">
-        <f>IF(OR(AND(E38&lt;&gt;"",NOT(ISNUMBER(E38)),E38&lt;&gt;"ABSENT"),AND(F38&lt;&gt;"",NOT(ISNUMBER(F38)),F38&lt;&gt;"ABSENT"),AND(G38&lt;&gt;"",NOT(ISNUMBER(G38)),G38&lt;&gt;"ABSENT"),AND(H38&lt;&gt;"",NOT(ISNUMBER(H38)),H38&lt;&gt;"ABSENT"),AND(ISNUMBER(E38),E38&lt;0),AND(ISNUMBER(F38),F38&lt;0),AND(ISNUMBER(G38),G38&lt;0),AND(ISNUMBER(H38),H38&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E38),E38&gt;E$4),AND(ISNUMBER(F38),F38&gt;F$4),AND(ISNUMBER(G38),G38&gt;G$4),AND(ISNUMBER(H38),H38&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G38),K38="still failed: presented from the executed notebook",G38&gt;=$G$4),"DEMO RULE",IF(COUNT(E38:H38)+COUNTIF(E38:H38,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E38="","GD ","")&amp;IF(F38="","group part ","")&amp;IF(G38="","presentation and defence ","")&amp;IF(H38="","mock","")),IF(COUNTIF(E38:H38,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E38="ABSENT","GD ","")&amp;IF(F38="ABSENT","group part ","")&amp;IF(G38="ABSENT","presentation and defence ","")&amp;IF(H38="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E38&lt;&gt;"",NOT(ISNUMBER(E38)),E38&lt;&gt;"ABSENT"),AND(F38&lt;&gt;"",NOT(ISNUMBER(F38)),F38&lt;&gt;"ABSENT"),AND(G38&lt;&gt;"",NOT(ISNUMBER(G38)),G38&lt;&gt;"ABSENT"),AND(H38&lt;&gt;"",NOT(ISNUMBER(H38)),H38&lt;&gt;"ABSENT"),AND(F38&lt;&gt;"",NOT(ISNUMBER(F38))),AND(ISNUMBER(E38),E38&lt;0),AND(ISNUMBER(F38),F38&lt;0),AND(ISNUMBER(G38),G38&lt;0),AND(ISNUMBER(H38),H38&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E38),E38&gt;E$4),AND(ISNUMBER(F38),F38&gt;F$4),AND(ISNUMBER(G38),G38&gt;G$4),AND(ISNUMBER(H38),H38&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F38),SUMPRODUCT(($B$6:$B$40=B38)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F38))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G38),K38="still failed: presented from the executed notebook",G38&gt;=$G$4),"DEMO RULE",IF(COUNT(E38:H38)+COUNTIF(E38:H38,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E38="","GD ","")&amp;IF(F38="","group part ","")&amp;IF(G38="","presentation and defence ","")&amp;IF(H38="","mock","")),IF(COUNTIF(E38:H38,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E38="ABSENT","GD ","")&amp;IF(F38="ABSENT","group part ","")&amp;IF(G38="ABSENT","presentation and defence ","")&amp;IF(H38="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M38" s="10" t="n"/>
@@ -2661,7 +2661,7 @@
         <v/>
       </c>
       <c r="L39" s="9">
-        <f>IF(OR(AND(E39&lt;&gt;"",NOT(ISNUMBER(E39)),E39&lt;&gt;"ABSENT"),AND(F39&lt;&gt;"",NOT(ISNUMBER(F39)),F39&lt;&gt;"ABSENT"),AND(G39&lt;&gt;"",NOT(ISNUMBER(G39)),G39&lt;&gt;"ABSENT"),AND(H39&lt;&gt;"",NOT(ISNUMBER(H39)),H39&lt;&gt;"ABSENT"),AND(ISNUMBER(E39),E39&lt;0),AND(ISNUMBER(F39),F39&lt;0),AND(ISNUMBER(G39),G39&lt;0),AND(ISNUMBER(H39),H39&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E39),E39&gt;E$4),AND(ISNUMBER(F39),F39&gt;F$4),AND(ISNUMBER(G39),G39&gt;G$4),AND(ISNUMBER(H39),H39&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G39),K39="still failed: presented from the executed notebook",G39&gt;=$G$4),"DEMO RULE",IF(COUNT(E39:H39)+COUNTIF(E39:H39,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E39="","GD ","")&amp;IF(F39="","group part ","")&amp;IF(G39="","presentation and defence ","")&amp;IF(H39="","mock","")),IF(COUNTIF(E39:H39,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E39="ABSENT","GD ","")&amp;IF(F39="ABSENT","group part ","")&amp;IF(G39="ABSENT","presentation and defence ","")&amp;IF(H39="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E39&lt;&gt;"",NOT(ISNUMBER(E39)),E39&lt;&gt;"ABSENT"),AND(F39&lt;&gt;"",NOT(ISNUMBER(F39)),F39&lt;&gt;"ABSENT"),AND(G39&lt;&gt;"",NOT(ISNUMBER(G39)),G39&lt;&gt;"ABSENT"),AND(H39&lt;&gt;"",NOT(ISNUMBER(H39)),H39&lt;&gt;"ABSENT"),AND(F39&lt;&gt;"",NOT(ISNUMBER(F39))),AND(ISNUMBER(E39),E39&lt;0),AND(ISNUMBER(F39),F39&lt;0),AND(ISNUMBER(G39),G39&lt;0),AND(ISNUMBER(H39),H39&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E39),E39&gt;E$4),AND(ISNUMBER(F39),F39&gt;F$4),AND(ISNUMBER(G39),G39&gt;G$4),AND(ISNUMBER(H39),H39&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F39),SUMPRODUCT(($B$6:$B$40=B39)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F39))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G39),K39="still failed: presented from the executed notebook",G39&gt;=$G$4),"DEMO RULE",IF(COUNT(E39:H39)+COUNTIF(E39:H39,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E39="","GD ","")&amp;IF(F39="","group part ","")&amp;IF(G39="","presentation and defence ","")&amp;IF(H39="","mock","")),IF(COUNTIF(E39:H39,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E39="ABSENT","GD ","")&amp;IF(F39="ABSENT","group part ","")&amp;IF(G39="ABSENT","presentation and defence ","")&amp;IF(H39="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M39" s="10" t="n"/>
@@ -2704,7 +2704,7 @@
         <v/>
       </c>
       <c r="L40" s="9">
-        <f>IF(OR(AND(E40&lt;&gt;"",NOT(ISNUMBER(E40)),E40&lt;&gt;"ABSENT"),AND(F40&lt;&gt;"",NOT(ISNUMBER(F40)),F40&lt;&gt;"ABSENT"),AND(G40&lt;&gt;"",NOT(ISNUMBER(G40)),G40&lt;&gt;"ABSENT"),AND(H40&lt;&gt;"",NOT(ISNUMBER(H40)),H40&lt;&gt;"ABSENT"),AND(ISNUMBER(E40),E40&lt;0),AND(ISNUMBER(F40),F40&lt;0),AND(ISNUMBER(G40),G40&lt;0),AND(ISNUMBER(H40),H40&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E40),E40&gt;E$4),AND(ISNUMBER(F40),F40&gt;F$4),AND(ISNUMBER(G40),G40&gt;G$4),AND(ISNUMBER(H40),H40&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(G40),K40="still failed: presented from the executed notebook",G40&gt;=$G$4),"DEMO RULE",IF(COUNT(E40:H40)+COUNTIF(E40:H40,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E40="","GD ","")&amp;IF(F40="","group part ","")&amp;IF(G40="","presentation and defence ","")&amp;IF(H40="","mock","")),IF(COUNTIF(E40:H40,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E40="ABSENT","GD ","")&amp;IF(F40="ABSENT","group part ","")&amp;IF(G40="ABSENT","presentation and defence ","")&amp;IF(H40="ABSENT","mock","")),"COMPLETE")))))</f>
+        <f>IF(OR(AND(E40&lt;&gt;"",NOT(ISNUMBER(E40)),E40&lt;&gt;"ABSENT"),AND(F40&lt;&gt;"",NOT(ISNUMBER(F40)),F40&lt;&gt;"ABSENT"),AND(G40&lt;&gt;"",NOT(ISNUMBER(G40)),G40&lt;&gt;"ABSENT"),AND(H40&lt;&gt;"",NOT(ISNUMBER(H40)),H40&lt;&gt;"ABSENT"),AND(F40&lt;&gt;"",NOT(ISNUMBER(F40))),AND(ISNUMBER(E40),E40&lt;0),AND(ISNUMBER(F40),F40&lt;0),AND(ISNUMBER(G40),G40&lt;0),AND(ISNUMBER(H40),H40&lt;0)),"NOT A SCORE",IF(OR(AND(ISNUMBER(E40),E40&gt;E$4),AND(ISNUMBER(F40),F40&gt;F$4),AND(ISNUMBER(G40),G40&gt;G$4),AND(ISNUMBER(H40),H40&gt;H$4)),"OVER MAX",IF(AND(ISNUMBER(F40),SUMPRODUCT(($B$6:$B$40=B40)*ISNUMBER($F$6:$F$40)*($F$6:$F$40&lt;&gt;F40))&gt;0),"GROUP PART DIFFERS",IF(AND(ISNUMBER(G40),K40="still failed: presented from the executed notebook",G40&gt;=$G$4),"DEMO RULE",IF(COUNT(E40:H40)+COUNTIF(E40:H40,"ABSENT")&lt;4,"MISSING "&amp;TRIM(IF(E40="","GD ","")&amp;IF(F40="","group part ","")&amp;IF(G40="","presentation and defence ","")&amp;IF(H40="","mock","")),IF(COUNTIF(E40:H40,"ABSENT")&gt;0,"ABSENT "&amp;TRIM(IF(E40="ABSENT","GD ","")&amp;IF(F40="ABSENT","group part ","")&amp;IF(G40="ABSENT","presentation and defence ","")&amp;IF(H40="ABSENT","mock","")),"COMPLETE"))))))</f>
         <v/>
       </c>
       <c r="M40" s="10" t="n"/>
@@ -3065,7 +3065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -3160,77 +3160,88 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Seats that break the DEMO RULE</t>
+          <t>Seats whose group part differs from a teammate's</t>
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Scores!$L$6:$L$40,"DEMO RULE")</f>
+        <f>COUNTIF(Scores!$L$6:$L$40,"GROUP PART DIFFERS")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Seats with an event marked ABSENT</t>
+          <t>Seats that break the DEMO RULE</t>
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Scores!$L$6:$L$40,"ABSENT*")</f>
+        <f>COUNTIF(Scores!$L$6:$L$40,"DEMO RULE")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Groups with a final demo outcome</t>
+          <t>Seats with an event marked ABSENT</t>
         </is>
       </c>
       <c r="B12" s="12">
-        <f>Demos!$B$14</f>
+        <f>COUNTIF(Scores!$L$6:$L$40,"ABSENT*")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Seats with no sub-problem or no panel recorded</t>
+          <t>Groups with a final demo outcome</t>
         </is>
       </c>
       <c r="B13" s="12">
-        <f>COUNTBLANK(Scores!$C$6:$C$40)+COUNTBLANK(Scores!$D$6:$D$40)</f>
+        <f>Demos!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Seats short, by seat</t>
-        </is>
-      </c>
-      <c r="B14" s="13">
-        <f>IF(LEN(Scores!N6&amp;Scores!N7&amp;Scores!N8&amp;Scores!N9&amp;Scores!N10&amp;Scores!N11&amp;Scores!N12&amp;Scores!N13&amp;Scores!N14&amp;Scores!N15&amp;Scores!N16&amp;Scores!N17&amp;Scores!N18&amp;Scores!N19&amp;Scores!N20&amp;Scores!N21&amp;Scores!N22&amp;Scores!N23&amp;Scores!N24&amp;Scores!N25&amp;Scores!N26&amp;Scores!N27&amp;Scores!N28&amp;Scores!N29&amp;Scores!N30&amp;Scores!N31&amp;Scores!N32&amp;Scores!N33&amp;Scores!N34&amp;Scores!N35&amp;Scores!N36&amp;Scores!N37&amp;Scores!N38&amp;Scores!N39&amp;Scores!N40)=0,"",LEFT(Scores!N6&amp;Scores!N7&amp;Scores!N8&amp;Scores!N9&amp;Scores!N10&amp;Scores!N11&amp;Scores!N12&amp;Scores!N13&amp;Scores!N14&amp;Scores!N15&amp;Scores!N16&amp;Scores!N17&amp;Scores!N18&amp;Scores!N19&amp;Scores!N20&amp;Scores!N21&amp;Scores!N22&amp;Scores!N23&amp;Scores!N24&amp;Scores!N25&amp;Scores!N26&amp;Scores!N27&amp;Scores!N28&amp;Scores!N29&amp;Scores!N30&amp;Scores!N31&amp;Scores!N32&amp;Scores!N33&amp;Scores!N34&amp;Scores!N35&amp;Scores!N36&amp;Scores!N37&amp;Scores!N38&amp;Scores!N39&amp;Scores!N40,LEN(Scores!N6&amp;Scores!N7&amp;Scores!N8&amp;Scores!N9&amp;Scores!N10&amp;Scores!N11&amp;Scores!N12&amp;Scores!N13&amp;Scores!N14&amp;Scores!N15&amp;Scores!N16&amp;Scores!N17&amp;Scores!N18&amp;Scores!N19&amp;Scores!N20&amp;Scores!N21&amp;Scores!N22&amp;Scores!N23&amp;Scores!N24&amp;Scores!N25&amp;Scores!N26&amp;Scores!N27&amp;Scores!N28&amp;Scores!N29&amp;Scores!N30&amp;Scores!N31&amp;Scores!N32&amp;Scores!N33&amp;Scores!N34&amp;Scores!N35&amp;Scores!N36&amp;Scores!N37&amp;Scores!N38&amp;Scores!N39&amp;Scores!N40)-2))</f>
+          <t>Seats with no sub-problem or no panel recorded</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>COUNTBLANK(Scores!$C$6:$C$40)+COUNTBLANK(Scores!$D$6:$D$40)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
+          <t>Seats short, by seat</t>
+        </is>
+      </c>
+      <c r="B15" s="13">
+        <f>IF(LEN(Scores!N6&amp;Scores!N7&amp;Scores!N8&amp;Scores!N9&amp;Scores!N10&amp;Scores!N11&amp;Scores!N12&amp;Scores!N13&amp;Scores!N14&amp;Scores!N15&amp;Scores!N16&amp;Scores!N17&amp;Scores!N18&amp;Scores!N19&amp;Scores!N20&amp;Scores!N21&amp;Scores!N22&amp;Scores!N23&amp;Scores!N24&amp;Scores!N25&amp;Scores!N26&amp;Scores!N27&amp;Scores!N28&amp;Scores!N29&amp;Scores!N30&amp;Scores!N31&amp;Scores!N32&amp;Scores!N33&amp;Scores!N34&amp;Scores!N35&amp;Scores!N36&amp;Scores!N37&amp;Scores!N38&amp;Scores!N39&amp;Scores!N40)=0,"",LEFT(Scores!N6&amp;Scores!N7&amp;Scores!N8&amp;Scores!N9&amp;Scores!N10&amp;Scores!N11&amp;Scores!N12&amp;Scores!N13&amp;Scores!N14&amp;Scores!N15&amp;Scores!N16&amp;Scores!N17&amp;Scores!N18&amp;Scores!N19&amp;Scores!N20&amp;Scores!N21&amp;Scores!N22&amp;Scores!N23&amp;Scores!N24&amp;Scores!N25&amp;Scores!N26&amp;Scores!N27&amp;Scores!N28&amp;Scores!N29&amp;Scores!N30&amp;Scores!N31&amp;Scores!N32&amp;Scores!N33&amp;Scores!N34&amp;Scores!N35&amp;Scores!N36&amp;Scores!N37&amp;Scores!N38&amp;Scores!N39&amp;Scores!N40,LEN(Scores!N6&amp;Scores!N7&amp;Scores!N8&amp;Scores!N9&amp;Scores!N10&amp;Scores!N11&amp;Scores!N12&amp;Scores!N13&amp;Scores!N14&amp;Scores!N15&amp;Scores!N16&amp;Scores!N17&amp;Scores!N18&amp;Scores!N19&amp;Scores!N20&amp;Scores!N21&amp;Scores!N22&amp;Scores!N23&amp;Scores!N24&amp;Scores!N25&amp;Scores!N26&amp;Scores!N27&amp;Scores!N28&amp;Scores!N29&amp;Scores!N30&amp;Scores!N31&amp;Scores!N32&amp;Scores!N33&amp;Scores!N34&amp;Scores!N35&amp;Scores!N36&amp;Scores!N37&amp;Scores!N38&amp;Scores!N39&amp;Scores!N40)-2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>Seats with an absence, by seat</t>
         </is>
       </c>
-      <c r="B15" s="13">
+      <c r="B16" s="13">
         <f>IF(LEN(Scores!O6&amp;Scores!O7&amp;Scores!O8&amp;Scores!O9&amp;Scores!O10&amp;Scores!O11&amp;Scores!O12&amp;Scores!O13&amp;Scores!O14&amp;Scores!O15&amp;Scores!O16&amp;Scores!O17&amp;Scores!O18&amp;Scores!O19&amp;Scores!O20&amp;Scores!O21&amp;Scores!O22&amp;Scores!O23&amp;Scores!O24&amp;Scores!O25&amp;Scores!O26&amp;Scores!O27&amp;Scores!O28&amp;Scores!O29&amp;Scores!O30&amp;Scores!O31&amp;Scores!O32&amp;Scores!O33&amp;Scores!O34&amp;Scores!O35&amp;Scores!O36&amp;Scores!O37&amp;Scores!O38&amp;Scores!O39&amp;Scores!O40)=0,"",LEFT(Scores!O6&amp;Scores!O7&amp;Scores!O8&amp;Scores!O9&amp;Scores!O10&amp;Scores!O11&amp;Scores!O12&amp;Scores!O13&amp;Scores!O14&amp;Scores!O15&amp;Scores!O16&amp;Scores!O17&amp;Scores!O18&amp;Scores!O19&amp;Scores!O20&amp;Scores!O21&amp;Scores!O22&amp;Scores!O23&amp;Scores!O24&amp;Scores!O25&amp;Scores!O26&amp;Scores!O27&amp;Scores!O28&amp;Scores!O29&amp;Scores!O30&amp;Scores!O31&amp;Scores!O32&amp;Scores!O33&amp;Scores!O34&amp;Scores!O35&amp;Scores!O36&amp;Scores!O37&amp;Scores!O38&amp;Scores!O39&amp;Scores!O40,LEN(Scores!O6&amp;Scores!O7&amp;Scores!O8&amp;Scores!O9&amp;Scores!O10&amp;Scores!O11&amp;Scores!O12&amp;Scores!O13&amp;Scores!O14&amp;Scores!O15&amp;Scores!O16&amp;Scores!O17&amp;Scores!O18&amp;Scores!O19&amp;Scores!O20&amp;Scores!O21&amp;Scores!O22&amp;Scores!O23&amp;Scores!O24&amp;Scores!O25&amp;Scores!O26&amp;Scores!O27&amp;Scores!O28&amp;Scores!O29&amp;Scores!O30&amp;Scores!O31&amp;Scores!O32&amp;Scores!O33&amp;Scores!O34&amp;Scores!O35&amp;Scores!O36&amp;Scores!O37&amp;Scores!O38&amp;Scores!O39&amp;Scores!O40)-2))</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="B17" s="15">
-        <f>IF(B4-B6-B11&gt;0,"NOT READY: "&amp;(B4-B6-B11)&amp;" seats short",IF(B5&gt;0,"NOT READY: a seat label repeats",IF(B12&lt;9,"NOT READY: record "&amp;(9-B12)&amp;" demo outcome(s)","READY TO SIGN")))</f>
+      <c r="B18" s="15">
+        <f>IF(B4-B6-B12&gt;0,"NOT READY: "&amp;(B4-B6-B12)&amp;" seats short",IF(B5&gt;0,"NOT READY: a seat label repeats",IF(B13&lt;9,"NOT READY: record "&amp;(9-B13)&amp;" demo outcome(s)","READY TO SIGN")))</f>
         <v/>
       </c>
     </row>
@@ -3402,7 +3413,7 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>IF(Checks!B17&lt;&gt;"READY TO SIGN","NOT READY",IF(COUNTIF(C4:C11,"Yes")=8,"CLOSED","READY: awaiting "&amp;(8-COUNTIF(C4:C11,"Yes"))&amp;" sign-offs"))</f>
+        <f>IF(Checks!B18&lt;&gt;"READY TO SIGN","NOT READY",IF(COUNTIF(C4:C11,"Yes")=8,"CLOSED","READY: awaiting "&amp;(8-COUNTIF(C4:C11,"Yes"))&amp;" sign-offs"))</f>
         <v/>
       </c>
     </row>

</xml_diff>